<commit_message>
📊 BIST Screener | 05.05.2026 16:30 | 610 hisse
</commit_message>
<xml_diff>
--- a/data/bist_screener_2026-05-05.xlsx
+++ b/data/bist_screener_2026-05-05.xlsx
@@ -18482,44 +18482,40 @@
     <row r="414">
       <c r="A414" s="2" t="inlineStr">
         <is>
-          <t>CCOLA</t>
+          <t>ARFYE</t>
         </is>
       </c>
       <c r="B414" s="3" t="n">
-        <v>79.84999999999999</v>
+        <v>33.04</v>
       </c>
       <c r="C414" s="4" t="n">
-        <v>0.039</v>
+        <v>0.0018</v>
       </c>
       <c r="D414" s="5" t="n">
-        <v>4940000</v>
+        <v>10660000</v>
       </c>
       <c r="E414" s="4" t="n">
-        <v>0.2895</v>
+        <v>0.2571</v>
       </c>
       <c r="F414" s="3" t="n">
-        <v>63.93</v>
-      </c>
-      <c r="G414" s="3" t="n">
-        <v>16.53</v>
-      </c>
+        <v>62.8</v>
+      </c>
+      <c r="G414" s="2" t="inlineStr"/>
       <c r="H414" s="3" t="n">
-        <v>2.95</v>
-      </c>
-      <c r="I414" s="4" t="n">
-        <v>0.2087</v>
-      </c>
+        <v>2.93</v>
+      </c>
+      <c r="I414" s="2" t="inlineStr"/>
       <c r="J414" s="4" t="n">
-        <v>-0.9989</v>
+        <v>-0.3467</v>
       </c>
       <c r="K414" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>Elektrik, Su, Gaz Hizmetleri</t>
         </is>
       </c>
       <c r="L414" s="2" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST GIDA ICECEK, BIST SINAI, BIST TÜM, BIST 50, BIST İSTANBUL, BIST 100-30, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST TEMETTU 25, BIST TEMETTU, BIST SÜRDÜRÜLEBİLİRLİK, BIST KURUMSAL YÖNETİM, BIST 50-30, BIST 50-30 AGIRLIK SINIRLAMALI 25, BIST 50-30 AĞIRLIK SINIRLAMALI 10, STOXX Emerging Markets 1500</t>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST KATILIM TÜM, BIST ANA, BIST İZMİR</t>
         </is>
       </c>
       <c r="M414" s="2" t="inlineStr"/>
@@ -18527,44 +18523,44 @@
     <row r="415">
       <c r="A415" s="6" t="inlineStr">
         <is>
-          <t>SUWEN</t>
+          <t>CCOLA</t>
         </is>
       </c>
       <c r="B415" s="7" t="n">
-        <v>8.69</v>
+        <v>79.84999999999999</v>
       </c>
       <c r="C415" s="8" t="n">
-        <v>0.008100000000000001</v>
+        <v>0.039</v>
       </c>
       <c r="D415" s="9" t="n">
-        <v>3210000</v>
+        <v>4940000</v>
       </c>
       <c r="E415" s="8" t="n">
-        <v>0.6501</v>
+        <v>0.2895</v>
       </c>
       <c r="F415" s="7" t="n">
-        <v>41.71</v>
+        <v>63.93</v>
       </c>
       <c r="G415" s="7" t="n">
-        <v>32.26</v>
+        <v>16.53</v>
       </c>
       <c r="H415" s="7" t="n">
         <v>2.95</v>
       </c>
       <c r="I415" s="8" t="n">
-        <v>0.078</v>
+        <v>0.2087</v>
       </c>
       <c r="J415" s="8" t="n">
-        <v>-0.9328</v>
+        <v>-0.9989</v>
       </c>
       <c r="K415" s="6" t="inlineStr">
         <is>
-          <t>Perakende satış</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L415" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST KATILIM TÜM, BIST YILDIZ, BIST TEMETTU, BIST KATILIM TEMETTU</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST GIDA ICECEK, BIST SINAI, BIST TÜM, BIST 50, BIST İSTANBUL, BIST 100-30, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST TEMETTU 25, BIST TEMETTU, BIST SÜRDÜRÜLEBİLİRLİK, BIST KURUMSAL YÖNETİM, BIST 50-30, BIST 50-30 AGIRLIK SINIRLAMALI 25, BIST 50-30 AĞIRLIK SINIRLAMALI 10, STOXX Emerging Markets 1500</t>
         </is>
       </c>
       <c r="M415" s="6" t="inlineStr"/>
@@ -18572,42 +18568,44 @@
     <row r="416">
       <c r="A416" s="2" t="inlineStr">
         <is>
-          <t>VBTYZ</t>
+          <t>SUWEN</t>
         </is>
       </c>
       <c r="B416" s="3" t="n">
-        <v>23.14</v>
+        <v>8.69</v>
       </c>
       <c r="C416" s="4" t="n">
-        <v>0.048</v>
+        <v>0.008100000000000001</v>
       </c>
       <c r="D416" s="5" t="n">
-        <v>1660000</v>
+        <v>3210000</v>
       </c>
       <c r="E416" s="4" t="n">
-        <v>0.371</v>
+        <v>0.6501</v>
       </c>
       <c r="F416" s="3" t="n">
-        <v>63.09</v>
+        <v>41.71</v>
       </c>
       <c r="G416" s="3" t="n">
-        <v>16.06</v>
+        <v>32.26</v>
       </c>
       <c r="H416" s="3" t="n">
-        <v>2.97</v>
+        <v>2.95</v>
       </c>
       <c r="I416" s="4" t="n">
-        <v>0.2008</v>
-      </c>
-      <c r="J416" s="2" t="inlineStr"/>
+        <v>0.078</v>
+      </c>
+      <c r="J416" s="4" t="n">
+        <v>-0.9328</v>
+      </c>
       <c r="K416" s="2" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
+          <t>Perakende satış</t>
         </is>
       </c>
       <c r="L416" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST KATILIM TÜM, BIST YILDIZ, BIST TEMETTU, BIST KATILIM TEMETTU</t>
         </is>
       </c>
       <c r="M416" s="2" t="inlineStr"/>
@@ -18615,44 +18613,42 @@
     <row r="417">
       <c r="A417" s="6" t="inlineStr">
         <is>
-          <t>TRALT</t>
+          <t>VBTYZ</t>
         </is>
       </c>
       <c r="B417" s="7" t="n">
-        <v>40.66</v>
+        <v>23.14</v>
       </c>
       <c r="C417" s="8" t="n">
-        <v>0.0283</v>
+        <v>0.048</v>
       </c>
       <c r="D417" s="9" t="n">
-        <v>113650000</v>
+        <v>1660000</v>
       </c>
       <c r="E417" s="8" t="n">
-        <v>0.3</v>
+        <v>0.371</v>
       </c>
       <c r="F417" s="7" t="n">
-        <v>37.77</v>
+        <v>63.09</v>
       </c>
       <c r="G417" s="7" t="n">
-        <v>33.06</v>
+        <v>16.06</v>
       </c>
       <c r="H417" s="7" t="n">
         <v>2.97</v>
       </c>
       <c r="I417" s="8" t="n">
-        <v>0.1092</v>
-      </c>
-      <c r="J417" s="8" t="n">
-        <v>-1.1669</v>
-      </c>
+        <v>0.2008</v>
+      </c>
+      <c r="J417" s="6" t="inlineStr"/>
       <c r="K417" s="6" t="inlineStr">
         <is>
-          <t>Enerji-dışı mineraller</t>
+          <t>Teknoloji hizmetleri</t>
         </is>
       </c>
       <c r="L417" s="6" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 30, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST SINAI, BIST TÜM, BIST MADENCİLİK, BIST 50, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST BANKA DISI LIKIT 10, BIST İZMİR, BIST 30 AĞIRLIK SINIRLAMALI 10, BIST 30 EŞİT AĞIRLIKLI GETİRİ, BIST 30 AĞIRLIK SINIRLAMALI 25, STOXX Emerging Markets 1500</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
         </is>
       </c>
       <c r="M417" s="6" t="inlineStr"/>
@@ -18660,44 +18656,44 @@
     <row r="418">
       <c r="A418" s="2" t="inlineStr">
         <is>
-          <t>FONET</t>
+          <t>TRALT</t>
         </is>
       </c>
       <c r="B418" s="3" t="n">
-        <v>5.48</v>
+        <v>40.66</v>
       </c>
       <c r="C418" s="4" t="n">
-        <v>0.0148</v>
+        <v>0.0283</v>
       </c>
       <c r="D418" s="5" t="n">
-        <v>67530000</v>
+        <v>113650000</v>
       </c>
       <c r="E418" s="4" t="n">
-        <v>0.6164999999999999</v>
+        <v>0.3</v>
       </c>
       <c r="F418" s="3" t="n">
-        <v>65.93000000000001</v>
+        <v>37.77</v>
       </c>
       <c r="G418" s="3" t="n">
-        <v>23.3</v>
+        <v>33.06</v>
       </c>
       <c r="H418" s="3" t="n">
-        <v>3.03</v>
+        <v>2.97</v>
       </c>
       <c r="I418" s="4" t="n">
-        <v>0.1565</v>
+        <v>0.1092</v>
       </c>
       <c r="J418" s="4" t="n">
-        <v>0.7060999999999999</v>
+        <v>-1.1669</v>
       </c>
       <c r="K418" s="2" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
+          <t>Enerji-dışı mineraller</t>
         </is>
       </c>
       <c r="L418" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST KATILIM 100, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST ANKARA</t>
+          <t>BIST 100, BIST 30, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST SINAI, BIST TÜM, BIST MADENCİLİK, BIST 50, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST BANKA DISI LIKIT 10, BIST İZMİR, BIST 30 AĞIRLIK SINIRLAMALI 10, BIST 30 EŞİT AĞIRLIKLI GETİRİ, BIST 30 AĞIRLIK SINIRLAMALI 25, STOXX Emerging Markets 1500</t>
         </is>
       </c>
       <c r="M418" s="2" t="inlineStr"/>
@@ -18705,42 +18701,44 @@
     <row r="419">
       <c r="A419" s="6" t="inlineStr">
         <is>
-          <t>KMPUR</t>
+          <t>FONET</t>
         </is>
       </c>
       <c r="B419" s="7" t="n">
-        <v>21.6</v>
+        <v>5.48</v>
       </c>
       <c r="C419" s="8" t="n">
-        <v>-0.0253</v>
+        <v>0.0148</v>
       </c>
       <c r="D419" s="9" t="n">
-        <v>6180000</v>
+        <v>67530000</v>
       </c>
       <c r="E419" s="8" t="n">
-        <v>0.1951</v>
+        <v>0.6164999999999999</v>
       </c>
       <c r="F419" s="7" t="n">
-        <v>71.09</v>
-      </c>
-      <c r="G419" s="6" t="inlineStr"/>
+        <v>65.93000000000001</v>
+      </c>
+      <c r="G419" s="7" t="n">
+        <v>23.3</v>
+      </c>
       <c r="H419" s="7" t="n">
-        <v>3.06</v>
+        <v>3.03</v>
       </c>
       <c r="I419" s="8" t="n">
-        <v>-0.098</v>
+        <v>0.1565</v>
       </c>
       <c r="J419" s="8" t="n">
-        <v>2.4746</v>
+        <v>0.7060999999999999</v>
       </c>
       <c r="K419" s="6" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Teknoloji hizmetleri</t>
         </is>
       </c>
       <c r="L419" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST KATILIM TÜM, BIST YILDIZ, BIST SÜRDÜRÜLEBİLİRLİK, BIST KURUMSAL YÖNETİM, BIST KOCAELI, BIST KATILIM SÜRDÜRÜLEBİLİRLİİK</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST KATILIM 100, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST ANKARA</t>
         </is>
       </c>
       <c r="M419" s="6" t="inlineStr"/>
@@ -18748,35 +18746,33 @@
     <row r="420">
       <c r="A420" s="2" t="inlineStr">
         <is>
-          <t>SAYAS</t>
+          <t>KMPUR</t>
         </is>
       </c>
       <c r="B420" s="3" t="n">
-        <v>49.7</v>
+        <v>21.6</v>
       </c>
       <c r="C420" s="4" t="n">
-        <v>-0.0442</v>
+        <v>-0.0253</v>
       </c>
       <c r="D420" s="5" t="n">
-        <v>2390000</v>
+        <v>6180000</v>
       </c>
       <c r="E420" s="4" t="n">
-        <v>0.5476</v>
+        <v>0.1951</v>
       </c>
       <c r="F420" s="3" t="n">
-        <v>63.74</v>
-      </c>
-      <c r="G420" s="3" t="n">
-        <v>25.33</v>
-      </c>
+        <v>71.09</v>
+      </c>
+      <c r="G420" s="2" t="inlineStr"/>
       <c r="H420" s="3" t="n">
-        <v>3.12</v>
+        <v>3.06</v>
       </c>
       <c r="I420" s="4" t="n">
-        <v>0.1475</v>
+        <v>-0.098</v>
       </c>
       <c r="J420" s="4" t="n">
-        <v>-0.7215</v>
+        <v>2.4746</v>
       </c>
       <c r="K420" s="2" t="inlineStr">
         <is>
@@ -18785,7 +18781,7 @@
       </c>
       <c r="L420" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST METAL ESYA MAKİNA, BIST KATILIM 100, BIST KATILIM TÜM, BIST ANA, BIST İZMİR</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST KATILIM TÜM, BIST YILDIZ, BIST SÜRDÜRÜLEBİLİRLİK, BIST KURUMSAL YÖNETİM, BIST KOCAELI, BIST KATILIM SÜRDÜRÜLEBİLİRLİİK</t>
         </is>
       </c>
       <c r="M420" s="2" t="inlineStr"/>
@@ -18793,42 +18789,44 @@
     <row r="421">
       <c r="A421" s="6" t="inlineStr">
         <is>
-          <t>AKSUE</t>
+          <t>SAYAS</t>
         </is>
       </c>
       <c r="B421" s="7" t="n">
-        <v>36.58</v>
+        <v>49.7</v>
       </c>
       <c r="C421" s="8" t="n">
-        <v>-0.0198</v>
+        <v>-0.0442</v>
       </c>
       <c r="D421" s="9" t="n">
-        <v>3280000</v>
+        <v>2390000</v>
       </c>
       <c r="E421" s="8" t="n">
-        <v>0.8798</v>
+        <v>0.5476</v>
       </c>
       <c r="F421" s="7" t="n">
-        <v>62.98</v>
-      </c>
-      <c r="G421" s="6" t="inlineStr"/>
+        <v>63.74</v>
+      </c>
+      <c r="G421" s="7" t="n">
+        <v>25.33</v>
+      </c>
       <c r="H421" s="7" t="n">
-        <v>3.17</v>
+        <v>3.12</v>
       </c>
       <c r="I421" s="8" t="n">
-        <v>-0.0545</v>
+        <v>0.1475</v>
       </c>
       <c r="J421" s="8" t="n">
-        <v>0.4473</v>
+        <v>-0.7215</v>
       </c>
       <c r="K421" s="6" t="inlineStr">
         <is>
-          <t>Elektrik, Su, Gaz Hizmetleri</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L421" s="6" t="inlineStr">
         <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST METAL ESYA MAKİNA, BIST KATILIM 100, BIST KATILIM TÜM, BIST ANA, BIST İZMİR</t>
         </is>
       </c>
       <c r="M421" s="6" t="inlineStr"/>
@@ -18836,33 +18834,33 @@
     <row r="422">
       <c r="A422" s="2" t="inlineStr">
         <is>
-          <t>TATEN</t>
+          <t>AKSUE</t>
         </is>
       </c>
       <c r="B422" s="3" t="n">
-        <v>15.43</v>
+        <v>36.58</v>
       </c>
       <c r="C422" s="4" t="n">
-        <v>0.0998</v>
+        <v>-0.0198</v>
       </c>
       <c r="D422" s="5" t="n">
-        <v>68520000</v>
+        <v>3280000</v>
       </c>
       <c r="E422" s="4" t="n">
-        <v>0.9165000000000001</v>
+        <v>0.8798</v>
       </c>
       <c r="F422" s="3" t="n">
-        <v>68.22</v>
+        <v>62.98</v>
       </c>
       <c r="G422" s="2" t="inlineStr"/>
       <c r="H422" s="3" t="n">
-        <v>3.22</v>
+        <v>3.17</v>
       </c>
       <c r="I422" s="4" t="n">
-        <v>-0.0159</v>
+        <v>-0.0545</v>
       </c>
       <c r="J422" s="4" t="n">
-        <v>-0.9540000000000001</v>
+        <v>0.4473</v>
       </c>
       <c r="K422" s="2" t="inlineStr">
         <is>
@@ -18871,7 +18869,7 @@
       </c>
       <c r="L422" s="2" t="inlineStr">
         <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST YILDIZ, BIST BALIKESİR</t>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST ANA</t>
         </is>
       </c>
       <c r="M422" s="2" t="inlineStr"/>
@@ -18879,33 +18877,33 @@
     <row r="423">
       <c r="A423" s="6" t="inlineStr">
         <is>
-          <t>BIGEN</t>
+          <t>TATEN</t>
         </is>
       </c>
       <c r="B423" s="7" t="n">
-        <v>18.48</v>
+        <v>15.43</v>
       </c>
       <c r="C423" s="8" t="n">
-        <v>-0.0999</v>
+        <v>0.0998</v>
       </c>
       <c r="D423" s="9" t="n">
-        <v>53040000</v>
+        <v>68520000</v>
       </c>
       <c r="E423" s="8" t="n">
-        <v>0.2002</v>
+        <v>0.9165000000000001</v>
       </c>
       <c r="F423" s="7" t="n">
-        <v>75.06999999999999</v>
+        <v>68.22</v>
       </c>
       <c r="G423" s="6" t="inlineStr"/>
       <c r="H423" s="7" t="n">
-        <v>3.23</v>
+        <v>3.22</v>
       </c>
       <c r="I423" s="8" t="n">
-        <v>-0.0906</v>
+        <v>-0.0159</v>
       </c>
       <c r="J423" s="8" t="n">
-        <v>-4.0218</v>
+        <v>-0.9540000000000001</v>
       </c>
       <c r="K423" s="6" t="inlineStr">
         <is>
@@ -18914,7 +18912,7 @@
       </c>
       <c r="L423" s="6" t="inlineStr">
         <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST YILDIZ, BIST BALIKESİR</t>
         </is>
       </c>
       <c r="M423" s="6" t="inlineStr"/>
@@ -18922,124 +18920,124 @@
     <row r="424">
       <c r="A424" s="2" t="inlineStr">
         <is>
-          <t>YBTAS</t>
+          <t>BIGEN</t>
         </is>
       </c>
       <c r="B424" s="3" t="n">
-        <v>17.64</v>
+        <v>18.48</v>
       </c>
       <c r="C424" s="4" t="n">
-        <v>0</v>
+        <v>-0.0999</v>
       </c>
       <c r="D424" s="5" t="n">
-        <v>105470</v>
+        <v>53040000</v>
       </c>
       <c r="E424" s="4" t="n">
-        <v>0.1931</v>
+        <v>0.2002</v>
       </c>
       <c r="F424" s="3" t="n">
-        <v>36.36</v>
+        <v>75.06999999999999</v>
       </c>
       <c r="G424" s="2" t="inlineStr"/>
       <c r="H424" s="3" t="n">
-        <v>3.24</v>
+        <v>3.23</v>
       </c>
       <c r="I424" s="4" t="n">
-        <v>-0.0482</v>
-      </c>
-      <c r="J424" s="2" t="inlineStr"/>
+        <v>-0.0906</v>
+      </c>
+      <c r="J424" s="4" t="n">
+        <v>-4.0218</v>
+      </c>
       <c r="K424" s="2" t="inlineStr">
         <is>
-          <t>Enerji-dışı mineraller</t>
-        </is>
-      </c>
-      <c r="L424" s="2" t="inlineStr"/>
+          <t>Elektrik, Su, Gaz Hizmetleri</t>
+        </is>
+      </c>
+      <c r="L424" s="2" t="inlineStr">
+        <is>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
+        </is>
+      </c>
       <c r="M424" s="2" t="inlineStr"/>
     </row>
     <row r="425">
       <c r="A425" s="6" t="inlineStr">
         <is>
-          <t>GIPTA</t>
+          <t>YBTAS</t>
         </is>
       </c>
       <c r="B425" s="7" t="n">
-        <v>81.40000000000001</v>
+        <v>17.64</v>
       </c>
       <c r="C425" s="8" t="n">
-        <v>-0.024</v>
+        <v>0</v>
       </c>
       <c r="D425" s="9" t="n">
-        <v>5770000</v>
+        <v>105470</v>
       </c>
       <c r="E425" s="8" t="n">
-        <v>0.3878</v>
+        <v>0.1931</v>
       </c>
       <c r="F425" s="7" t="n">
-        <v>54.84</v>
-      </c>
-      <c r="G425" s="7" t="n">
-        <v>54.17</v>
-      </c>
+        <v>36.36</v>
+      </c>
+      <c r="G425" s="6" t="inlineStr"/>
       <c r="H425" s="7" t="n">
         <v>3.24</v>
       </c>
       <c r="I425" s="8" t="n">
-        <v>0.0682</v>
-      </c>
-      <c r="J425" s="8" t="n">
-        <v>-2.8727</v>
-      </c>
+        <v>-0.0482</v>
+      </c>
+      <c r="J425" s="6" t="inlineStr"/>
       <c r="K425" s="6" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
-        </is>
-      </c>
-      <c r="L425" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST YILDIZ, BIST ANKARA</t>
-        </is>
-      </c>
+          <t>Enerji-dışı mineraller</t>
+        </is>
+      </c>
+      <c r="L425" s="6" t="inlineStr"/>
       <c r="M425" s="6" t="inlineStr"/>
     </row>
     <row r="426">
       <c r="A426" s="2" t="inlineStr">
         <is>
-          <t>DERIM</t>
+          <t>GIPTA</t>
         </is>
       </c>
       <c r="B426" s="3" t="n">
-        <v>37.78</v>
+        <v>81.40000000000001</v>
       </c>
       <c r="C426" s="4" t="n">
-        <v>0.0266</v>
+        <v>-0.024</v>
       </c>
       <c r="D426" s="5" t="n">
-        <v>530800</v>
-      </c>
-      <c r="E426" s="2" t="inlineStr"/>
+        <v>5770000</v>
+      </c>
+      <c r="E426" s="4" t="n">
+        <v>0.3878</v>
+      </c>
       <c r="F426" s="3" t="n">
-        <v>48.9</v>
+        <v>54.84</v>
       </c>
       <c r="G426" s="3" t="n">
-        <v>22.66</v>
+        <v>54.17</v>
       </c>
       <c r="H426" s="3" t="n">
         <v>3.24</v>
       </c>
       <c r="I426" s="4" t="n">
-        <v>0.1732</v>
+        <v>0.0682</v>
       </c>
       <c r="J426" s="4" t="n">
-        <v>8.039199999999999</v>
+        <v>-2.8727</v>
       </c>
       <c r="K426" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L426" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TEKSTİL DERİ, BIST İSTANBUL, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST YILDIZ, BIST ANKARA</t>
         </is>
       </c>
       <c r="M426" s="2" t="inlineStr"/>
@@ -19047,44 +19045,42 @@
     <row r="427">
       <c r="A427" s="6" t="inlineStr">
         <is>
-          <t>PATEK</t>
+          <t>DERIM</t>
         </is>
       </c>
       <c r="B427" s="7" t="n">
-        <v>22.96</v>
+        <v>37.78</v>
       </c>
       <c r="C427" s="8" t="n">
-        <v>0.09960000000000001</v>
+        <v>0.0266</v>
       </c>
       <c r="D427" s="9" t="n">
-        <v>16410000</v>
-      </c>
-      <c r="E427" s="8" t="n">
-        <v>0.4408</v>
-      </c>
+        <v>530800</v>
+      </c>
+      <c r="E427" s="6" t="inlineStr"/>
       <c r="F427" s="7" t="n">
-        <v>67.70999999999999</v>
+        <v>48.9</v>
       </c>
       <c r="G427" s="7" t="n">
-        <v>12.32</v>
+        <v>22.66</v>
       </c>
       <c r="H427" s="7" t="n">
-        <v>3.25</v>
+        <v>3.24</v>
       </c>
       <c r="I427" s="8" t="n">
-        <v>0.454</v>
+        <v>0.1732</v>
       </c>
       <c r="J427" s="8" t="n">
-        <v>-0.7884</v>
+        <v>8.039199999999999</v>
       </c>
       <c r="K427" s="6" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L427" s="6" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST 100-30, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TEKSTİL DERİ, BIST İSTANBUL, BIST ANA</t>
         </is>
       </c>
       <c r="M427" s="6" t="inlineStr"/>
@@ -19092,42 +19088,44 @@
     <row r="428">
       <c r="A428" s="2" t="inlineStr">
         <is>
-          <t>GMTAS</t>
+          <t>PATEK</t>
         </is>
       </c>
       <c r="B428" s="3" t="n">
-        <v>41.7</v>
+        <v>22.96</v>
       </c>
       <c r="C428" s="4" t="n">
-        <v>0.0296</v>
+        <v>0.09960000000000001</v>
       </c>
       <c r="D428" s="5" t="n">
-        <v>9200000</v>
+        <v>16410000</v>
       </c>
       <c r="E428" s="4" t="n">
-        <v>0.9993000000000001</v>
+        <v>0.4408</v>
       </c>
       <c r="F428" s="3" t="n">
-        <v>59.64</v>
-      </c>
-      <c r="G428" s="2" t="inlineStr"/>
+        <v>67.70999999999999</v>
+      </c>
+      <c r="G428" s="3" t="n">
+        <v>12.32</v>
+      </c>
       <c r="H428" s="3" t="n">
         <v>3.25</v>
       </c>
       <c r="I428" s="4" t="n">
-        <v>-0.0423</v>
+        <v>0.454</v>
       </c>
       <c r="J428" s="4" t="n">
-        <v>0.1053</v>
+        <v>-0.7884</v>
       </c>
       <c r="K428" s="2" t="inlineStr">
         <is>
-          <t>Perakende satış</t>
+          <t>Teknoloji hizmetleri</t>
         </is>
       </c>
       <c r="L428" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST KATILIM TÜM, BIST YILDIZ</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST 100-30, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
         </is>
       </c>
       <c r="M428" s="2" t="inlineStr"/>
@@ -19135,44 +19133,42 @@
     <row r="429">
       <c r="A429" s="6" t="inlineStr">
         <is>
-          <t>OZSUB</t>
+          <t>GMTAS</t>
         </is>
       </c>
       <c r="B429" s="7" t="n">
-        <v>28</v>
+        <v>41.7</v>
       </c>
       <c r="C429" s="8" t="n">
-        <v>-0.0237</v>
+        <v>0.0296</v>
       </c>
       <c r="D429" s="9" t="n">
-        <v>7620000</v>
+        <v>9200000</v>
       </c>
       <c r="E429" s="8" t="n">
-        <v>0.3082</v>
+        <v>0.9993000000000001</v>
       </c>
       <c r="F429" s="7" t="n">
-        <v>71.25</v>
-      </c>
-      <c r="G429" s="7" t="n">
-        <v>11.46</v>
-      </c>
+        <v>59.64</v>
+      </c>
+      <c r="G429" s="6" t="inlineStr"/>
       <c r="H429" s="7" t="n">
-        <v>3.26</v>
+        <v>3.25</v>
       </c>
       <c r="I429" s="8" t="n">
-        <v>0.3585</v>
+        <v>-0.0423</v>
       </c>
       <c r="J429" s="8" t="n">
-        <v>-0.5128</v>
+        <v>0.1053</v>
       </c>
       <c r="K429" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Perakende satış</t>
         </is>
       </c>
       <c r="L429" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ANA, BIST İZMİR</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST KATILIM TÜM, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M429" s="6" t="inlineStr"/>
@@ -19180,40 +19176,44 @@
     <row r="430">
       <c r="A430" s="2" t="inlineStr">
         <is>
-          <t>SMRTG</t>
+          <t>OZSUB</t>
         </is>
       </c>
       <c r="B430" s="3" t="n">
-        <v>8.359999999999999</v>
+        <v>28</v>
       </c>
       <c r="C430" s="4" t="n">
-        <v>0.0609</v>
-      </c>
-      <c r="D430" s="3" t="n">
-        <v>33230000</v>
+        <v>-0.0237</v>
+      </c>
+      <c r="D430" s="5" t="n">
+        <v>7620000</v>
       </c>
       <c r="E430" s="4" t="n">
-        <v>0.3655</v>
+        <v>0.3082</v>
       </c>
       <c r="F430" s="3" t="n">
-        <v>66.5</v>
-      </c>
-      <c r="G430" s="2" t="inlineStr"/>
+        <v>71.25</v>
+      </c>
+      <c r="G430" s="3" t="n">
+        <v>11.46</v>
+      </c>
       <c r="H430" s="3" t="n">
-        <v>3.28</v>
+        <v>3.26</v>
       </c>
       <c r="I430" s="4" t="n">
-        <v>-0.09390000000000001</v>
-      </c>
-      <c r="J430" s="2" t="inlineStr"/>
+        <v>0.3585</v>
+      </c>
+      <c r="J430" s="4" t="n">
+        <v>-0.5128</v>
+      </c>
       <c r="K430" s="2" t="inlineStr">
         <is>
-          <t>Elektronik teknoloji</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L430" s="2" t="inlineStr">
         <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST YILDIZ, BIST SÜRDÜRÜLEBİLİRLİK, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ANA, BIST İZMİR</t>
         </is>
       </c>
       <c r="M430" s="2" t="inlineStr"/>
@@ -19221,42 +19221,40 @@
     <row r="431">
       <c r="A431" s="6" t="inlineStr">
         <is>
-          <t>LINK</t>
+          <t>SMRTG</t>
         </is>
       </c>
       <c r="B431" s="7" t="n">
-        <v>6.01</v>
+        <v>8.359999999999999</v>
       </c>
       <c r="C431" s="8" t="n">
-        <v>0.0169</v>
-      </c>
-      <c r="D431" s="9" t="n">
-        <v>43240000</v>
+        <v>0.0609</v>
+      </c>
+      <c r="D431" s="7" t="n">
+        <v>33230000</v>
       </c>
       <c r="E431" s="8" t="n">
-        <v>0.9937</v>
+        <v>0.3655</v>
       </c>
       <c r="F431" s="7" t="n">
-        <v>64.3</v>
-      </c>
-      <c r="G431" s="7" t="n">
-        <v>17.52</v>
-      </c>
+        <v>66.5</v>
+      </c>
+      <c r="G431" s="6" t="inlineStr"/>
       <c r="H431" s="7" t="n">
-        <v>3.3</v>
+        <v>3.28</v>
       </c>
       <c r="I431" s="8" t="n">
-        <v>0.2337</v>
+        <v>-0.09390000000000001</v>
       </c>
       <c r="J431" s="6" t="inlineStr"/>
       <c r="K431" s="6" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
+          <t>Elektronik teknoloji</t>
         </is>
       </c>
       <c r="L431" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST YILDIZ, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST YILDIZ, BIST SÜRDÜRÜLEBİLİRLİK, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M431" s="6" t="inlineStr"/>
@@ -19264,44 +19262,42 @@
     <row r="432">
       <c r="A432" s="2" t="inlineStr">
         <is>
-          <t>GRTHO</t>
+          <t>LINK</t>
         </is>
       </c>
       <c r="B432" s="3" t="n">
-        <v>245.2</v>
+        <v>6.01</v>
       </c>
       <c r="C432" s="4" t="n">
-        <v>-0.0089</v>
+        <v>0.0169</v>
       </c>
       <c r="D432" s="5" t="n">
-        <v>1320000</v>
+        <v>43240000</v>
       </c>
       <c r="E432" s="4" t="n">
-        <v>0.29</v>
+        <v>0.9937</v>
       </c>
       <c r="F432" s="3" t="n">
-        <v>47.86</v>
+        <v>64.3</v>
       </c>
       <c r="G432" s="3" t="n">
-        <v>17.48</v>
+        <v>17.52</v>
       </c>
       <c r="H432" s="3" t="n">
-        <v>3.4</v>
+        <v>3.3</v>
       </c>
       <c r="I432" s="4" t="n">
-        <v>0.248</v>
-      </c>
-      <c r="J432" s="4" t="n">
-        <v>1.037</v>
-      </c>
+        <v>0.2337</v>
+      </c>
+      <c r="J432" s="2" t="inlineStr"/>
       <c r="K432" s="2" t="inlineStr">
         <is>
-          <t>Dağıtım servisleri</t>
+          <t>Teknoloji hizmetleri</t>
         </is>
       </c>
       <c r="L432" s="2" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST İSTANBUL, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST YILDIZ, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
         </is>
       </c>
       <c r="M432" s="2" t="inlineStr"/>
@@ -19309,42 +19305,44 @@
     <row r="433">
       <c r="A433" s="6" t="inlineStr">
         <is>
-          <t>GZNMI</t>
+          <t>GRTHO</t>
         </is>
       </c>
       <c r="B433" s="7" t="n">
-        <v>72.40000000000001</v>
+        <v>245.2</v>
       </c>
       <c r="C433" s="8" t="n">
-        <v>0.0343</v>
+        <v>-0.0089</v>
       </c>
       <c r="D433" s="9" t="n">
-        <v>5680000</v>
+        <v>1320000</v>
       </c>
       <c r="E433" s="8" t="n">
-        <v>0.3987</v>
+        <v>0.29</v>
       </c>
       <c r="F433" s="7" t="n">
-        <v>53.85</v>
-      </c>
-      <c r="G433" s="6" t="inlineStr"/>
+        <v>47.86</v>
+      </c>
+      <c r="G433" s="7" t="n">
+        <v>17.48</v>
+      </c>
       <c r="H433" s="7" t="n">
-        <v>3.45</v>
+        <v>3.4</v>
       </c>
       <c r="I433" s="8" t="n">
-        <v>-0.0958</v>
+        <v>0.248</v>
       </c>
       <c r="J433" s="8" t="n">
-        <v>-2.2418</v>
+        <v>1.037</v>
       </c>
       <c r="K433" s="6" t="inlineStr">
         <is>
-          <t>Tüketici hizmetleri</t>
+          <t>Dağıtım servisleri</t>
         </is>
       </c>
       <c r="L433" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST ANA, BIST ANTALYA</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST İSTANBUL, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50</t>
         </is>
       </c>
       <c r="M433" s="6" t="inlineStr"/>
@@ -19352,44 +19350,42 @@
     <row r="434">
       <c r="A434" s="2" t="inlineStr">
         <is>
-          <t>ATATP</t>
+          <t>GZNMI</t>
         </is>
       </c>
       <c r="B434" s="3" t="n">
-        <v>162.3</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="C434" s="4" t="n">
-        <v>0.0351</v>
+        <v>0.0343</v>
       </c>
       <c r="D434" s="5" t="n">
-        <v>1170000</v>
+        <v>5680000</v>
       </c>
       <c r="E434" s="4" t="n">
-        <v>0.0158</v>
+        <v>0.3987</v>
       </c>
       <c r="F434" s="3" t="n">
-        <v>66.45</v>
-      </c>
-      <c r="G434" s="3" t="n">
-        <v>2.15</v>
-      </c>
+        <v>53.85</v>
+      </c>
+      <c r="G434" s="2" t="inlineStr"/>
       <c r="H434" s="3" t="n">
         <v>3.45</v>
       </c>
       <c r="I434" s="4" t="n">
-        <v>0.6533</v>
+        <v>-0.0958</v>
       </c>
       <c r="J434" s="4" t="n">
-        <v>-0.1442</v>
+        <v>-2.2418</v>
       </c>
       <c r="K434" s="2" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
+          <t>Tüketici hizmetleri</t>
         </is>
       </c>
       <c r="L434" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST ANA, BIST ANTALYA</t>
         </is>
       </c>
       <c r="M434" s="2" t="inlineStr"/>
@@ -19397,44 +19393,44 @@
     <row r="435">
       <c r="A435" s="6" t="inlineStr">
         <is>
-          <t>RAYSG</t>
+          <t>ATATP</t>
         </is>
       </c>
       <c r="B435" s="7" t="n">
-        <v>198.9</v>
+        <v>162.3</v>
       </c>
       <c r="C435" s="8" t="n">
-        <v>0.0311</v>
+        <v>0.0351</v>
       </c>
       <c r="D435" s="9" t="n">
-        <v>252700</v>
+        <v>1170000</v>
       </c>
       <c r="E435" s="8" t="n">
-        <v>0.0504</v>
+        <v>0.0158</v>
       </c>
       <c r="F435" s="7" t="n">
-        <v>47.26</v>
+        <v>66.45</v>
       </c>
       <c r="G435" s="7" t="n">
-        <v>8.449999999999999</v>
+        <v>2.15</v>
       </c>
       <c r="H435" s="7" t="n">
-        <v>3.47</v>
+        <v>3.45</v>
       </c>
       <c r="I435" s="8" t="n">
-        <v>0.5283</v>
+        <v>0.6533</v>
       </c>
       <c r="J435" s="8" t="n">
-        <v>0.6009</v>
+        <v>-0.1442</v>
       </c>
       <c r="K435" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Teknoloji hizmetleri</t>
         </is>
       </c>
       <c r="L435" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST SİGORTA, BIST MALİ, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
         </is>
       </c>
       <c r="M435" s="6" t="inlineStr"/>
@@ -19442,42 +19438,44 @@
     <row r="436">
       <c r="A436" s="2" t="inlineStr">
         <is>
-          <t>IZINV</t>
+          <t>RAYSG</t>
         </is>
       </c>
       <c r="B436" s="3" t="n">
-        <v>72</v>
+        <v>198.9</v>
       </c>
       <c r="C436" s="4" t="n">
-        <v>-0.027</v>
+        <v>0.0311</v>
       </c>
       <c r="D436" s="5" t="n">
-        <v>1120000</v>
+        <v>252700</v>
       </c>
       <c r="E436" s="4" t="n">
-        <v>0.7040999999999999</v>
+        <v>0.0504</v>
       </c>
       <c r="F436" s="3" t="n">
-        <v>57</v>
-      </c>
-      <c r="G436" s="2" t="inlineStr"/>
+        <v>47.26</v>
+      </c>
+      <c r="G436" s="3" t="n">
+        <v>8.449999999999999</v>
+      </c>
       <c r="H436" s="3" t="n">
-        <v>3.53</v>
+        <v>3.47</v>
       </c>
       <c r="I436" s="4" t="n">
-        <v>-0.1552</v>
+        <v>0.5283</v>
       </c>
       <c r="J436" s="4" t="n">
-        <v>-0.45</v>
+        <v>0.6009</v>
       </c>
       <c r="K436" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L436" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST KOBİ SANAYİ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST SİGORTA, BIST MALİ, BIST ANA</t>
         </is>
       </c>
       <c r="M436" s="2" t="inlineStr"/>
@@ -19485,44 +19483,42 @@
     <row r="437">
       <c r="A437" s="6" t="inlineStr">
         <is>
-          <t>TCKRC</t>
+          <t>IZINV</t>
         </is>
       </c>
       <c r="B437" s="7" t="n">
-        <v>110</v>
+        <v>72</v>
       </c>
       <c r="C437" s="8" t="n">
-        <v>-0.0161</v>
+        <v>-0.027</v>
       </c>
       <c r="D437" s="9" t="n">
-        <v>5500000</v>
+        <v>1120000</v>
       </c>
       <c r="E437" s="8" t="n">
-        <v>0.3229</v>
+        <v>0.7040999999999999</v>
       </c>
       <c r="F437" s="7" t="n">
-        <v>69.45999999999999</v>
-      </c>
-      <c r="G437" s="7" t="n">
-        <v>15.49</v>
-      </c>
+        <v>57</v>
+      </c>
+      <c r="G437" s="6" t="inlineStr"/>
       <c r="H437" s="7" t="n">
-        <v>3.56</v>
+        <v>3.53</v>
       </c>
       <c r="I437" s="8" t="n">
-        <v>0.2909</v>
+        <v>-0.1552</v>
       </c>
       <c r="J437" s="8" t="n">
-        <v>2.7171</v>
+        <v>-0.45</v>
       </c>
       <c r="K437" s="6" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L437" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST METAL ANA, BIST HALKA ARZ, BIST YILDIZ, BIST BURSA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST KOBİ SANAYİ</t>
         </is>
       </c>
       <c r="M437" s="6" t="inlineStr"/>
@@ -19530,35 +19526,35 @@
     <row r="438">
       <c r="A438" s="2" t="inlineStr">
         <is>
-          <t>KBORU</t>
+          <t>TCKRC</t>
         </is>
       </c>
       <c r="B438" s="3" t="n">
-        <v>26.82</v>
+        <v>110</v>
       </c>
       <c r="C438" s="4" t="n">
-        <v>0.004500000000000001</v>
+        <v>-0.0161</v>
       </c>
       <c r="D438" s="5" t="n">
-        <v>14650000</v>
+        <v>5500000</v>
       </c>
       <c r="E438" s="4" t="n">
-        <v>0.24</v>
+        <v>0.3229</v>
       </c>
       <c r="F438" s="3" t="n">
-        <v>75.19</v>
+        <v>69.45999999999999</v>
       </c>
       <c r="G438" s="3" t="n">
-        <v>27.31</v>
+        <v>15.49</v>
       </c>
       <c r="H438" s="3" t="n">
-        <v>3.62</v>
+        <v>3.56</v>
       </c>
       <c r="I438" s="4" t="n">
-        <v>0.1577</v>
+        <v>0.2909</v>
       </c>
       <c r="J438" s="4" t="n">
-        <v>0.8172</v>
+        <v>2.7171</v>
       </c>
       <c r="K438" s="2" t="inlineStr">
         <is>
@@ -19567,7 +19563,7 @@
       </c>
       <c r="L438" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST KATILIM 100, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST METAL ANA, BIST HALKA ARZ, BIST YILDIZ, BIST BURSA</t>
         </is>
       </c>
       <c r="M438" s="2" t="inlineStr"/>
@@ -19575,42 +19571,44 @@
     <row r="439">
       <c r="A439" s="6" t="inlineStr">
         <is>
-          <t>KARTN</t>
+          <t>KBORU</t>
         </is>
       </c>
       <c r="B439" s="7" t="n">
-        <v>119.7</v>
+        <v>26.82</v>
       </c>
       <c r="C439" s="8" t="n">
-        <v>0.0992</v>
+        <v>0.004500000000000001</v>
       </c>
       <c r="D439" s="9" t="n">
-        <v>2320000</v>
+        <v>14650000</v>
       </c>
       <c r="E439" s="8" t="n">
-        <v>0.2186</v>
+        <v>0.24</v>
       </c>
       <c r="F439" s="7" t="n">
-        <v>73.88</v>
-      </c>
-      <c r="G439" s="6" t="inlineStr"/>
+        <v>75.19</v>
+      </c>
+      <c r="G439" s="7" t="n">
+        <v>27.31</v>
+      </c>
       <c r="H439" s="7" t="n">
-        <v>3.63</v>
+        <v>3.62</v>
       </c>
       <c r="I439" s="8" t="n">
-        <v>-0.4183</v>
+        <v>0.1577</v>
       </c>
       <c r="J439" s="8" t="n">
-        <v>-1.6177</v>
+        <v>0.8172</v>
       </c>
       <c r="K439" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L439" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST ANA, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST KATILIM 100, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M439" s="6" t="inlineStr"/>
@@ -19618,33 +19616,33 @@
     <row r="440">
       <c r="A440" s="2" t="inlineStr">
         <is>
-          <t>BARMA</t>
+          <t>KARTN</t>
         </is>
       </c>
       <c r="B440" s="3" t="n">
-        <v>60.05</v>
+        <v>119.7</v>
       </c>
       <c r="C440" s="4" t="n">
-        <v>-0.0066</v>
+        <v>0.0992</v>
       </c>
       <c r="D440" s="5" t="n">
-        <v>1770000</v>
+        <v>2320000</v>
       </c>
       <c r="E440" s="4" t="n">
-        <v>0.2</v>
+        <v>0.2186</v>
       </c>
       <c r="F440" s="3" t="n">
-        <v>71.05</v>
+        <v>73.88</v>
       </c>
       <c r="G440" s="2" t="inlineStr"/>
       <c r="H440" s="3" t="n">
         <v>3.63</v>
       </c>
       <c r="I440" s="4" t="n">
-        <v>-0.005600000000000001</v>
+        <v>-0.4183</v>
       </c>
       <c r="J440" s="4" t="n">
-        <v>-0.7101999999999999</v>
+        <v>-1.6177</v>
       </c>
       <c r="K440" s="2" t="inlineStr">
         <is>
@@ -19653,7 +19651,7 @@
       </c>
       <c r="L440" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST YILDIZ, BIST İZMİR</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M440" s="2" t="inlineStr"/>
@@ -19661,44 +19659,42 @@
     <row r="441">
       <c r="A441" s="6" t="inlineStr">
         <is>
-          <t>EUPWR</t>
+          <t>BARMA</t>
         </is>
       </c>
       <c r="B441" s="7" t="n">
-        <v>58.8</v>
+        <v>60.05</v>
       </c>
       <c r="C441" s="8" t="n">
-        <v>0.0604</v>
+        <v>-0.0066</v>
       </c>
       <c r="D441" s="9" t="n">
-        <v>32790000</v>
+        <v>1770000</v>
       </c>
       <c r="E441" s="8" t="n">
-        <v>0.3025</v>
+        <v>0.2</v>
       </c>
       <c r="F441" s="7" t="n">
-        <v>82.19</v>
-      </c>
-      <c r="G441" s="7" t="n">
-        <v>67.7</v>
-      </c>
+        <v>71.05</v>
+      </c>
+      <c r="G441" s="6" t="inlineStr"/>
       <c r="H441" s="7" t="n">
-        <v>3.68</v>
+        <v>3.63</v>
       </c>
       <c r="I441" s="8" t="n">
-        <v>0.06320000000000001</v>
+        <v>-0.005600000000000001</v>
       </c>
       <c r="J441" s="8" t="n">
-        <v>-1.0812</v>
+        <v>-0.7101999999999999</v>
       </c>
       <c r="K441" s="6" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L441" s="6" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST SINAI, BIST TÜM, BIST METAL ESYA MAKİNA, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST YILDIZ, BIST İZMİR</t>
         </is>
       </c>
       <c r="M441" s="6" t="inlineStr"/>
@@ -19706,42 +19702,44 @@
     <row r="442">
       <c r="A442" s="2" t="inlineStr">
         <is>
-          <t>ALTNY</t>
+          <t>EUPWR</t>
         </is>
       </c>
       <c r="B442" s="3" t="n">
-        <v>17.02</v>
+        <v>58.8</v>
       </c>
       <c r="C442" s="4" t="n">
-        <v>0.0296</v>
+        <v>0.0604</v>
       </c>
       <c r="D442" s="5" t="n">
-        <v>28050000</v>
+        <v>32790000</v>
       </c>
       <c r="E442" s="4" t="n">
-        <v>0.3999</v>
+        <v>0.3025</v>
       </c>
       <c r="F442" s="3" t="n">
-        <v>67.3</v>
+        <v>82.19</v>
       </c>
       <c r="G442" s="3" t="n">
-        <v>69.84</v>
+        <v>67.7</v>
       </c>
       <c r="H442" s="3" t="n">
         <v>3.68</v>
       </c>
       <c r="I442" s="4" t="n">
-        <v>-0.0039</v>
-      </c>
-      <c r="J442" s="2" t="inlineStr"/>
+        <v>0.06320000000000001</v>
+      </c>
+      <c r="J442" s="4" t="n">
+        <v>-1.0812</v>
+      </c>
       <c r="K442" s="2" t="inlineStr">
         <is>
-          <t>Elektronik teknoloji</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L442" s="2" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST TEKNOLOJİ, BIST HALKA ARZ, BIST İSTANBUL, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM 30, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST SINAI, BIST TÜM, BIST METAL ESYA MAKİNA, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
         </is>
       </c>
       <c r="M442" s="2" t="inlineStr"/>
@@ -19749,42 +19747,42 @@
     <row r="443">
       <c r="A443" s="6" t="inlineStr">
         <is>
-          <t>MIATK</t>
+          <t>ALTNY</t>
         </is>
       </c>
       <c r="B443" s="7" t="n">
-        <v>40.8</v>
+        <v>17.02</v>
       </c>
       <c r="C443" s="8" t="n">
-        <v>0.044</v>
+        <v>0.0296</v>
       </c>
       <c r="D443" s="9" t="n">
-        <v>19240000</v>
+        <v>28050000</v>
       </c>
       <c r="E443" s="8" t="n">
-        <v>0.5778</v>
+        <v>0.3999</v>
       </c>
       <c r="F443" s="7" t="n">
-        <v>53.18</v>
-      </c>
-      <c r="G443" s="6" t="inlineStr"/>
+        <v>67.3</v>
+      </c>
+      <c r="G443" s="7" t="n">
+        <v>69.84</v>
+      </c>
       <c r="H443" s="7" t="n">
-        <v>3.69</v>
+        <v>3.68</v>
       </c>
       <c r="I443" s="8" t="n">
-        <v>-0.1487</v>
-      </c>
-      <c r="J443" s="8" t="n">
-        <v>0.5216</v>
-      </c>
+        <v>-0.0039</v>
+      </c>
+      <c r="J443" s="6" t="inlineStr"/>
       <c r="K443" s="6" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
+          <t>Elektronik teknoloji</t>
         </is>
       </c>
       <c r="L443" s="6" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST 50, BIST 100-30, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST 50-30, BIST ANKARA, BIST 50-30 AGIRLIK SINIRLAMALI 25, BIST 50-30 AĞIRLIK SINIRLAMALI 10</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST TEKNOLOJİ, BIST HALKA ARZ, BIST İSTANBUL, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM 30, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
         </is>
       </c>
       <c r="M443" s="6" t="inlineStr"/>
@@ -19792,35 +19790,33 @@
     <row r="444">
       <c r="A444" s="2" t="inlineStr">
         <is>
-          <t>ARDYZ</t>
+          <t>MIATK</t>
         </is>
       </c>
       <c r="B444" s="3" t="n">
-        <v>58</v>
+        <v>40.8</v>
       </c>
       <c r="C444" s="4" t="n">
-        <v>0.0507</v>
+        <v>0.044</v>
       </c>
       <c r="D444" s="5" t="n">
-        <v>6990000</v>
+        <v>19240000</v>
       </c>
       <c r="E444" s="4" t="n">
-        <v>0.3949</v>
+        <v>0.5778</v>
       </c>
       <c r="F444" s="3" t="n">
-        <v>81.04000000000001</v>
-      </c>
-      <c r="G444" s="3" t="n">
-        <v>27.7</v>
-      </c>
+        <v>53.18</v>
+      </c>
+      <c r="G444" s="2" t="inlineStr"/>
       <c r="H444" s="3" t="n">
-        <v>3.7</v>
+        <v>3.69</v>
       </c>
       <c r="I444" s="4" t="n">
-        <v>0.1333</v>
+        <v>-0.1487</v>
       </c>
       <c r="J444" s="4" t="n">
-        <v>6.844600000000001</v>
+        <v>0.5216</v>
       </c>
       <c r="K444" s="2" t="inlineStr">
         <is>
@@ -19829,7 +19825,7 @@
       </c>
       <c r="L444" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST 50, BIST 100-30, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST 50-30, BIST ANKARA, BIST 50-30 AGIRLIK SINIRLAMALI 25, BIST 50-30 AĞIRLIK SINIRLAMALI 10</t>
         </is>
       </c>
       <c r="M444" s="2" t="inlineStr"/>
@@ -19837,44 +19833,44 @@
     <row r="445">
       <c r="A445" s="6" t="inlineStr">
         <is>
-          <t>EGEGY</t>
+          <t>ARDYZ</t>
         </is>
       </c>
       <c r="B445" s="7" t="n">
-        <v>31.8</v>
+        <v>58</v>
       </c>
       <c r="C445" s="8" t="n">
-        <v>0.0127</v>
+        <v>0.0507</v>
       </c>
       <c r="D445" s="9" t="n">
-        <v>3900000</v>
+        <v>6990000</v>
       </c>
       <c r="E445" s="8" t="n">
-        <v>0.306</v>
+        <v>0.3949</v>
       </c>
       <c r="F445" s="7" t="n">
-        <v>57.8</v>
+        <v>81.04000000000001</v>
       </c>
       <c r="G445" s="7" t="n">
-        <v>8.130000000000001</v>
+        <v>27.7</v>
       </c>
       <c r="H445" s="7" t="n">
-        <v>3.71</v>
+        <v>3.7</v>
       </c>
       <c r="I445" s="8" t="n">
-        <v>0.8473999999999999</v>
+        <v>0.1333</v>
       </c>
       <c r="J445" s="8" t="n">
-        <v>5.585199999999999</v>
+        <v>6.844600000000001</v>
       </c>
       <c r="K445" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Teknoloji hizmetleri</t>
         </is>
       </c>
       <c r="L445" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
         </is>
       </c>
       <c r="M445" s="6" t="inlineStr"/>
@@ -19882,42 +19878,44 @@
     <row r="446">
       <c r="A446" s="2" t="inlineStr">
         <is>
-          <t>EMKEL</t>
+          <t>EGEGY</t>
         </is>
       </c>
       <c r="B446" s="3" t="n">
-        <v>24.74</v>
+        <v>31.8</v>
       </c>
       <c r="C446" s="4" t="n">
-        <v>0.009000000000000001</v>
+        <v>0.0127</v>
       </c>
       <c r="D446" s="5" t="n">
-        <v>27120000</v>
+        <v>3900000</v>
       </c>
       <c r="E446" s="4" t="n">
-        <v>0.9773999999999999</v>
+        <v>0.306</v>
       </c>
       <c r="F446" s="3" t="n">
-        <v>49.76</v>
-      </c>
-      <c r="G446" s="2" t="inlineStr"/>
+        <v>57.8</v>
+      </c>
+      <c r="G446" s="3" t="n">
+        <v>8.130000000000001</v>
+      </c>
       <c r="H446" s="3" t="n">
-        <v>3.79</v>
+        <v>3.71</v>
       </c>
       <c r="I446" s="4" t="n">
-        <v>-0.0576</v>
+        <v>0.8473999999999999</v>
       </c>
       <c r="J446" s="4" t="n">
-        <v>-2.2771</v>
+        <v>5.585199999999999</v>
       </c>
       <c r="K446" s="2" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L446" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST METAL ESYA MAKİNA, BIST ANA, BIST ANKARA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST ANA</t>
         </is>
       </c>
       <c r="M446" s="2" t="inlineStr"/>
@@ -19925,42 +19923,42 @@
     <row r="447">
       <c r="A447" s="6" t="inlineStr">
         <is>
-          <t>BIOEN</t>
+          <t>EMKEL</t>
         </is>
       </c>
       <c r="B447" s="7" t="n">
-        <v>21.3</v>
+        <v>24.74</v>
       </c>
       <c r="C447" s="8" t="n">
-        <v>0.0513</v>
+        <v>0.009000000000000001</v>
       </c>
       <c r="D447" s="9" t="n">
-        <v>12890000</v>
+        <v>27120000</v>
       </c>
       <c r="E447" s="8" t="n">
-        <v>0.3959</v>
+        <v>0.9773999999999999</v>
       </c>
       <c r="F447" s="7" t="n">
-        <v>68.86</v>
+        <v>49.76</v>
       </c>
       <c r="G447" s="6" t="inlineStr"/>
       <c r="H447" s="7" t="n">
-        <v>3.82</v>
+        <v>3.79</v>
       </c>
       <c r="I447" s="8" t="n">
-        <v>-0.3911</v>
+        <v>-0.0576</v>
       </c>
       <c r="J447" s="8" t="n">
-        <v>-4.4402</v>
+        <v>-2.2771</v>
       </c>
       <c r="K447" s="6" t="inlineStr">
         <is>
-          <t>Elektrik, Su, Gaz Hizmetleri</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L447" s="6" t="inlineStr">
         <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST YILDIZ, BIST SÜRDÜRÜLEBİLİRLİK, BIST KURUMSAL YÖNETİM, BIST İZMİR</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST METAL ESYA MAKİNA, BIST ANA, BIST ANKARA</t>
         </is>
       </c>
       <c r="M447" s="6" t="inlineStr"/>
@@ -19968,44 +19966,42 @@
     <row r="448">
       <c r="A448" s="2" t="inlineStr">
         <is>
-          <t>GENIL</t>
+          <t>BIOEN</t>
         </is>
       </c>
       <c r="B448" s="3" t="n">
-        <v>8.880000000000001</v>
+        <v>21.3</v>
       </c>
       <c r="C448" s="4" t="n">
-        <v>-0.0022</v>
+        <v>0.0513</v>
       </c>
       <c r="D448" s="5" t="n">
-        <v>29710000</v>
+        <v>12890000</v>
       </c>
       <c r="E448" s="4" t="n">
-        <v>0.2412</v>
+        <v>0.3959</v>
       </c>
       <c r="F448" s="3" t="n">
-        <v>33.54</v>
-      </c>
-      <c r="G448" s="3" t="n">
-        <v>52.24</v>
-      </c>
+        <v>68.86</v>
+      </c>
+      <c r="G448" s="2" t="inlineStr"/>
       <c r="H448" s="3" t="n">
-        <v>3.86</v>
+        <v>3.82</v>
       </c>
       <c r="I448" s="4" t="n">
-        <v>0.0866</v>
+        <v>-0.3911</v>
       </c>
       <c r="J448" s="4" t="n">
-        <v>-0.3022</v>
+        <v>-4.4402</v>
       </c>
       <c r="K448" s="2" t="inlineStr">
         <is>
-          <t>Sağlık teknolojisi</t>
+          <t>Elektrik, Su, Gaz Hizmetleri</t>
         </is>
       </c>
       <c r="L448" s="2" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST TEMETTU, BIST KATILIM 50, BIST KATILIM 30, BIST KATILIM TEMETTU, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST YILDIZ, BIST SÜRDÜRÜLEBİLİRLİK, BIST KURUMSAL YÖNETİM, BIST İZMİR</t>
         </is>
       </c>
       <c r="M448" s="2" t="inlineStr"/>
@@ -20013,44 +20009,44 @@
     <row r="449">
       <c r="A449" s="6" t="inlineStr">
         <is>
-          <t>LOGO</t>
+          <t>GENIL</t>
         </is>
       </c>
       <c r="B449" s="7" t="n">
-        <v>153.1</v>
+        <v>8.880000000000001</v>
       </c>
       <c r="C449" s="8" t="n">
-        <v>0.031</v>
+        <v>-0.0022</v>
       </c>
       <c r="D449" s="9" t="n">
-        <v>931540</v>
+        <v>29710000</v>
       </c>
       <c r="E449" s="8" t="n">
-        <v>0.6459999999999999</v>
+        <v>0.2412</v>
       </c>
       <c r="F449" s="7" t="n">
-        <v>68.66</v>
+        <v>33.54</v>
       </c>
       <c r="G449" s="7" t="n">
-        <v>10.48</v>
+        <v>52.24</v>
       </c>
       <c r="H449" s="7" t="n">
-        <v>3.89</v>
+        <v>3.86</v>
       </c>
       <c r="I449" s="8" t="n">
-        <v>0.4715</v>
+        <v>0.0866</v>
       </c>
       <c r="J449" s="8" t="n">
-        <v>-0.4521</v>
+        <v>-0.3022</v>
       </c>
       <c r="K449" s="6" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
+          <t>Sağlık teknolojisi</t>
         </is>
       </c>
       <c r="L449" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST SÜRDÜRÜLEBİLİRLİK, BIST KURUMSAL YÖNETİM, BIST KATILIM TEMETTU, BIST KOCAELI, BIST KATILIM SÜRDÜRÜLEBİLİRLİİK</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST TEMETTU, BIST KATILIM 50, BIST KATILIM 30, BIST KATILIM TEMETTU, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
         </is>
       </c>
       <c r="M449" s="6" t="inlineStr"/>
@@ -20058,42 +20054,44 @@
     <row r="450">
       <c r="A450" s="2" t="inlineStr">
         <is>
-          <t>TARKM</t>
+          <t>LOGO</t>
         </is>
       </c>
       <c r="B450" s="3" t="n">
-        <v>469</v>
+        <v>153.1</v>
       </c>
       <c r="C450" s="4" t="n">
-        <v>0.0434</v>
+        <v>0.031</v>
       </c>
       <c r="D450" s="5" t="n">
-        <v>311410</v>
+        <v>931540</v>
       </c>
       <c r="E450" s="4" t="n">
-        <v>0.2381</v>
+        <v>0.6459999999999999</v>
       </c>
       <c r="F450" s="3" t="n">
-        <v>75.76000000000001</v>
-      </c>
-      <c r="G450" s="2" t="inlineStr"/>
+        <v>68.66</v>
+      </c>
+      <c r="G450" s="3" t="n">
+        <v>10.48</v>
+      </c>
       <c r="H450" s="3" t="n">
-        <v>3.94</v>
+        <v>3.89</v>
       </c>
       <c r="I450" s="4" t="n">
-        <v>-0.0599</v>
+        <v>0.4715</v>
       </c>
       <c r="J450" s="4" t="n">
-        <v>-44.8491</v>
+        <v>-0.4521</v>
       </c>
       <c r="K450" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Teknoloji hizmetleri</t>
         </is>
       </c>
       <c r="L450" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST KATILIM 100, BIST KATILIM TÜM, BIST ANA, BIST MANİSA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST SÜRDÜRÜLEBİLİRLİK, BIST KURUMSAL YÖNETİM, BIST KATILIM TEMETTU, BIST KOCAELI, BIST KATILIM SÜRDÜRÜLEBİLİRLİİK</t>
         </is>
       </c>
       <c r="M450" s="2" t="inlineStr"/>
@@ -20101,33 +20099,33 @@
     <row r="451">
       <c r="A451" s="6" t="inlineStr">
         <is>
-          <t>ALKA</t>
+          <t>TARKM</t>
         </is>
       </c>
       <c r="B451" s="7" t="n">
-        <v>11.44</v>
+        <v>469</v>
       </c>
       <c r="C451" s="8" t="n">
-        <v>0.0467</v>
+        <v>0.0434</v>
       </c>
       <c r="D451" s="9" t="n">
-        <v>8100000</v>
+        <v>311410</v>
       </c>
       <c r="E451" s="8" t="n">
-        <v>0.1937</v>
+        <v>0.2381</v>
       </c>
       <c r="F451" s="7" t="n">
-        <v>50.77</v>
+        <v>75.76000000000001</v>
       </c>
       <c r="G451" s="6" t="inlineStr"/>
       <c r="H451" s="7" t="n">
-        <v>4.04</v>
+        <v>3.94</v>
       </c>
       <c r="I451" s="8" t="n">
-        <v>-0.0556</v>
+        <v>-0.0599</v>
       </c>
       <c r="J451" s="8" t="n">
-        <v>-7.241000000000001</v>
+        <v>-44.8491</v>
       </c>
       <c r="K451" s="6" t="inlineStr">
         <is>
@@ -20136,7 +20134,7 @@
       </c>
       <c r="L451" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST KATILIM TÜM, BIST ANA, BIST İZMİR</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST KATILIM 100, BIST KATILIM TÜM, BIST ANA, BIST MANİSA</t>
         </is>
       </c>
       <c r="M451" s="6" t="inlineStr"/>
@@ -20144,33 +20142,33 @@
     <row r="452">
       <c r="A452" s="2" t="inlineStr">
         <is>
-          <t>OTTO</t>
+          <t>ALKA</t>
         </is>
       </c>
       <c r="B452" s="3" t="n">
-        <v>301.25</v>
+        <v>11.44</v>
       </c>
       <c r="C452" s="4" t="n">
-        <v>-0.0066</v>
+        <v>0.0467</v>
       </c>
       <c r="D452" s="5" t="n">
-        <v>473510</v>
+        <v>8100000</v>
       </c>
       <c r="E452" s="4" t="n">
-        <v>0.3623</v>
+        <v>0.1937</v>
       </c>
       <c r="F452" s="3" t="n">
-        <v>36.22</v>
+        <v>50.77</v>
       </c>
       <c r="G452" s="2" t="inlineStr"/>
       <c r="H452" s="3" t="n">
         <v>4.04</v>
       </c>
       <c r="I452" s="4" t="n">
-        <v>-0.0108</v>
+        <v>-0.0556</v>
       </c>
       <c r="J452" s="4" t="n">
-        <v>-0.3881</v>
+        <v>-7.241000000000001</v>
       </c>
       <c r="K452" s="2" t="inlineStr">
         <is>
@@ -20179,7 +20177,7 @@
       </c>
       <c r="L452" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST İSTANBUL, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST KATILIM TÜM, BIST ANA, BIST İZMİR</t>
         </is>
       </c>
       <c r="M452" s="2" t="inlineStr"/>
@@ -20187,42 +20185,42 @@
     <row r="453">
       <c r="A453" s="6" t="inlineStr">
         <is>
-          <t>BURCE</t>
+          <t>OTTO</t>
         </is>
       </c>
       <c r="B453" s="7" t="n">
-        <v>53.25</v>
+        <v>301.25</v>
       </c>
       <c r="C453" s="8" t="n">
-        <v>-0.044</v>
+        <v>-0.0066</v>
       </c>
       <c r="D453" s="9" t="n">
-        <v>10750000</v>
+        <v>473510</v>
       </c>
       <c r="E453" s="8" t="n">
-        <v>0.5275</v>
+        <v>0.3623</v>
       </c>
       <c r="F453" s="7" t="n">
-        <v>53.94</v>
+        <v>36.22</v>
       </c>
       <c r="G453" s="6" t="inlineStr"/>
       <c r="H453" s="7" t="n">
-        <v>4.06</v>
+        <v>4.04</v>
       </c>
       <c r="I453" s="8" t="n">
-        <v>-0.1171</v>
+        <v>-0.0108</v>
       </c>
       <c r="J453" s="8" t="n">
-        <v>-1.2976</v>
+        <v>-0.3881</v>
       </c>
       <c r="K453" s="6" t="inlineStr">
         <is>
-          <t>Enerji-dışı mineraller</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L453" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST METAL ANA, BIST KATILIM TÜM, BIST ANA, BIST BURSA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST İSTANBUL, BIST ANA</t>
         </is>
       </c>
       <c r="M453" s="6" t="inlineStr"/>
@@ -20230,44 +20228,42 @@
     <row r="454">
       <c r="A454" s="2" t="inlineStr">
         <is>
-          <t>AGESA</t>
+          <t>BURCE</t>
         </is>
       </c>
       <c r="B454" s="3" t="n">
-        <v>236.3</v>
+        <v>53.25</v>
       </c>
       <c r="C454" s="4" t="n">
-        <v>-0.0113</v>
+        <v>-0.044</v>
       </c>
       <c r="D454" s="5" t="n">
-        <v>213600</v>
+        <v>10750000</v>
       </c>
       <c r="E454" s="4" t="n">
-        <v>0.2</v>
+        <v>0.5275</v>
       </c>
       <c r="F454" s="3" t="n">
-        <v>54.04</v>
-      </c>
-      <c r="G454" s="3" t="n">
-        <v>6.94</v>
-      </c>
+        <v>53.94</v>
+      </c>
+      <c r="G454" s="2" t="inlineStr"/>
       <c r="H454" s="3" t="n">
         <v>4.06</v>
       </c>
       <c r="I454" s="4" t="n">
-        <v>0.7723</v>
+        <v>-0.1171</v>
       </c>
       <c r="J454" s="4" t="n">
-        <v>0.2044</v>
+        <v>-1.2976</v>
       </c>
       <c r="K454" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Enerji-dışı mineraller</t>
         </is>
       </c>
       <c r="L454" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST SİGORTA, BIST MALİ, BIST YILDIZ, BIST TEMETTU, BIST SÜRDÜRÜLEBİLİRLİK</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST METAL ANA, BIST KATILIM TÜM, BIST ANA, BIST BURSA</t>
         </is>
       </c>
       <c r="M454" s="2" t="inlineStr"/>
@@ -20275,42 +20271,44 @@
     <row r="455">
       <c r="A455" s="6" t="inlineStr">
         <is>
-          <t>PAMEL</t>
+          <t>AGESA</t>
         </is>
       </c>
       <c r="B455" s="7" t="n">
-        <v>90</v>
+        <v>236.3</v>
       </c>
       <c r="C455" s="8" t="n">
-        <v>-0.0323</v>
+        <v>-0.0113</v>
       </c>
       <c r="D455" s="9" t="n">
-        <v>666750</v>
+        <v>213600</v>
       </c>
       <c r="E455" s="8" t="n">
-        <v>0.2393</v>
+        <v>0.2</v>
       </c>
       <c r="F455" s="7" t="n">
-        <v>54.74</v>
-      </c>
-      <c r="G455" s="6" t="inlineStr"/>
+        <v>54.04</v>
+      </c>
+      <c r="G455" s="7" t="n">
+        <v>6.94</v>
+      </c>
       <c r="H455" s="7" t="n">
-        <v>4.15</v>
+        <v>4.06</v>
       </c>
       <c r="I455" s="8" t="n">
-        <v>-0.4116</v>
+        <v>0.7723</v>
       </c>
       <c r="J455" s="8" t="n">
-        <v>-8.8185</v>
+        <v>0.2044</v>
       </c>
       <c r="K455" s="6" t="inlineStr">
         <is>
-          <t>Elektrik, Su, Gaz Hizmetleri</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L455" s="6" t="inlineStr">
         <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST SİGORTA, BIST MALİ, BIST YILDIZ, BIST TEMETTU, BIST SÜRDÜRÜLEBİLİRLİK</t>
         </is>
       </c>
       <c r="M455" s="6" t="inlineStr"/>
@@ -20318,40 +20316,42 @@
     <row r="456">
       <c r="A456" s="2" t="inlineStr">
         <is>
-          <t>EUYO</t>
+          <t>PAMEL</t>
         </is>
       </c>
       <c r="B456" s="3" t="n">
-        <v>5.54</v>
+        <v>90</v>
       </c>
       <c r="C456" s="4" t="n">
-        <v>-0.0195</v>
+        <v>-0.0323</v>
       </c>
       <c r="D456" s="5" t="n">
-        <v>879360</v>
-      </c>
-      <c r="E456" s="2" t="inlineStr"/>
+        <v>666750</v>
+      </c>
+      <c r="E456" s="4" t="n">
+        <v>0.2393</v>
+      </c>
       <c r="F456" s="3" t="n">
-        <v>39.63</v>
+        <v>54.74</v>
       </c>
       <c r="G456" s="2" t="inlineStr"/>
       <c r="H456" s="3" t="n">
-        <v>4.18</v>
+        <v>4.15</v>
       </c>
       <c r="I456" s="4" t="n">
-        <v>-0.2073</v>
+        <v>-0.4116</v>
       </c>
       <c r="J456" s="4" t="n">
-        <v>-2.3315</v>
+        <v>-8.8185</v>
       </c>
       <c r="K456" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Elektrik, Su, Gaz Hizmetleri</t>
         </is>
       </c>
       <c r="L456" s="2" t="inlineStr">
         <is>
-          <t>BIST MENKUL KIYM YO</t>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST ANA</t>
         </is>
       </c>
       <c r="M456" s="2" t="inlineStr"/>
@@ -20359,44 +20359,40 @@
     <row r="457">
       <c r="A457" s="6" t="inlineStr">
         <is>
-          <t>SAFKR</t>
+          <t>EUYO</t>
         </is>
       </c>
       <c r="B457" s="7" t="n">
-        <v>24.34</v>
+        <v>5.54</v>
       </c>
       <c r="C457" s="8" t="n">
-        <v>0.0411</v>
+        <v>-0.0195</v>
       </c>
       <c r="D457" s="9" t="n">
-        <v>5770000</v>
-      </c>
-      <c r="E457" s="8" t="n">
-        <v>0.6303</v>
-      </c>
+        <v>879360</v>
+      </c>
+      <c r="E457" s="6" t="inlineStr"/>
       <c r="F457" s="7" t="n">
-        <v>40.8</v>
-      </c>
-      <c r="G457" s="7" t="n">
-        <v>30.05</v>
-      </c>
+        <v>39.63</v>
+      </c>
+      <c r="G457" s="6" t="inlineStr"/>
       <c r="H457" s="7" t="n">
         <v>4.18</v>
       </c>
       <c r="I457" s="8" t="n">
-        <v>0.1679</v>
+        <v>-0.2073</v>
       </c>
       <c r="J457" s="8" t="n">
-        <v>0.2955</v>
+        <v>-2.3315</v>
       </c>
       <c r="K457" s="6" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L457" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST METAL ESYA MAKİNA, BIST KATILIM 100, BIST KATILIM TÜM, BIST ANA, BIST İZMİR</t>
+          <t>BIST MENKUL KIYM YO</t>
         </is>
       </c>
       <c r="M457" s="6" t="inlineStr"/>
@@ -20404,44 +20400,44 @@
     <row r="458">
       <c r="A458" s="2" t="inlineStr">
         <is>
-          <t>DOCO</t>
-        </is>
-      </c>
-      <c r="B458" s="5" t="n">
-        <v>8875</v>
+          <t>SAFKR</t>
+        </is>
+      </c>
+      <c r="B458" s="3" t="n">
+        <v>24.34</v>
       </c>
       <c r="C458" s="4" t="n">
-        <v>-0.004500000000000001</v>
+        <v>0.0411</v>
       </c>
       <c r="D458" s="5" t="n">
-        <v>9510</v>
+        <v>5770000</v>
       </c>
       <c r="E458" s="4" t="n">
-        <v>0.6981000000000001</v>
+        <v>0.6303</v>
       </c>
       <c r="F458" s="3" t="n">
-        <v>42.93</v>
+        <v>40.8</v>
       </c>
       <c r="G458" s="3" t="n">
-        <v>18.25</v>
+        <v>30.05</v>
       </c>
       <c r="H458" s="3" t="n">
-        <v>4.23</v>
+        <v>4.18</v>
       </c>
       <c r="I458" s="4" t="n">
-        <v>0.2552</v>
+        <v>0.1679</v>
       </c>
       <c r="J458" s="4" t="n">
-        <v>0.2085</v>
+        <v>0.2955</v>
       </c>
       <c r="K458" s="2" t="inlineStr">
         <is>
-          <t>Tüketici hizmetleri</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L458" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TURİZM, BIST HİZMETLER, BIST ANA, BIST SÜRDÜRÜLEBİLİRLİK</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST METAL ESYA MAKİNA, BIST KATILIM 100, BIST KATILIM TÜM, BIST ANA, BIST İZMİR</t>
         </is>
       </c>
       <c r="M458" s="2" t="inlineStr"/>
@@ -20449,44 +20445,44 @@
     <row r="459">
       <c r="A459" s="6" t="inlineStr">
         <is>
-          <t>ANHYT</t>
-        </is>
-      </c>
-      <c r="B459" s="7" t="n">
-        <v>112.9</v>
+          <t>DOCO</t>
+        </is>
+      </c>
+      <c r="B459" s="9" t="n">
+        <v>8875</v>
       </c>
       <c r="C459" s="8" t="n">
-        <v>0.0236</v>
+        <v>-0.004500000000000001</v>
       </c>
       <c r="D459" s="9" t="n">
-        <v>863780</v>
+        <v>9510</v>
       </c>
       <c r="E459" s="8" t="n">
-        <v>0.1508</v>
+        <v>0.6981000000000001</v>
       </c>
       <c r="F459" s="7" t="n">
-        <v>52.11</v>
+        <v>42.93</v>
       </c>
       <c r="G459" s="7" t="n">
-        <v>7.47</v>
+        <v>18.25</v>
       </c>
       <c r="H459" s="7" t="n">
-        <v>4.28</v>
+        <v>4.23</v>
       </c>
       <c r="I459" s="8" t="n">
-        <v>0.6579999999999999</v>
+        <v>0.2552</v>
       </c>
       <c r="J459" s="8" t="n">
-        <v>-0.1602</v>
+        <v>0.2085</v>
       </c>
       <c r="K459" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Tüketici hizmetleri</t>
         </is>
       </c>
       <c r="L459" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST SİGORTA, BIST MALİ, BIST YILDIZ, BIST TEMETTU 25, BIST TEMETTU, BIST SÜRDÜRÜLEBİLİRLİK</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TURİZM, BIST HİZMETLER, BIST ANA, BIST SÜRDÜRÜLEBİLİRLİK</t>
         </is>
       </c>
       <c r="M459" s="6" t="inlineStr"/>
@@ -20494,44 +20490,44 @@
     <row r="460">
       <c r="A460" s="2" t="inlineStr">
         <is>
-          <t>HTTBT</t>
+          <t>ANHYT</t>
         </is>
       </c>
       <c r="B460" s="3" t="n">
-        <v>42.5</v>
+        <v>112.9</v>
       </c>
       <c r="C460" s="4" t="n">
-        <v>0.03759999999999999</v>
+        <v>0.0236</v>
       </c>
       <c r="D460" s="5" t="n">
-        <v>789610</v>
+        <v>863780</v>
       </c>
       <c r="E460" s="4" t="n">
-        <v>0.276</v>
+        <v>0.1508</v>
       </c>
       <c r="F460" s="3" t="n">
-        <v>57.5</v>
+        <v>52.11</v>
       </c>
       <c r="G460" s="3" t="n">
-        <v>32.79</v>
+        <v>7.47</v>
       </c>
       <c r="H460" s="3" t="n">
-        <v>4.3</v>
+        <v>4.28</v>
       </c>
       <c r="I460" s="4" t="n">
-        <v>0.1536</v>
+        <v>0.6579999999999999</v>
       </c>
       <c r="J460" s="4" t="n">
-        <v>-0.1008</v>
+        <v>-0.1602</v>
       </c>
       <c r="K460" s="2" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L460" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST YILDIZ, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST SÜRDÜRÜLEBİLİRLİK, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST TÜM, BIST SİGORTA, BIST MALİ, BIST YILDIZ, BIST TEMETTU 25, BIST TEMETTU, BIST SÜRDÜRÜLEBİLİRLİK</t>
         </is>
       </c>
       <c r="M460" s="2" t="inlineStr"/>
@@ -20539,122 +20535,124 @@
     <row r="461">
       <c r="A461" s="6" t="inlineStr">
         <is>
-          <t>SUMAS</t>
+          <t>HTTBT</t>
         </is>
       </c>
       <c r="B461" s="7" t="n">
-        <v>349.25</v>
+        <v>42.5</v>
       </c>
       <c r="C461" s="8" t="n">
-        <v>0.1</v>
+        <v>0.03759999999999999</v>
       </c>
       <c r="D461" s="9" t="n">
-        <v>8880</v>
+        <v>789610</v>
       </c>
       <c r="E461" s="8" t="n">
-        <v>0.3229</v>
+        <v>0.276</v>
       </c>
       <c r="F461" s="7" t="n">
-        <v>81.84999999999999</v>
+        <v>57.5</v>
       </c>
       <c r="G461" s="7" t="n">
-        <v>135.22</v>
+        <v>32.79</v>
       </c>
       <c r="H461" s="7" t="n">
-        <v>4.31</v>
+        <v>4.3</v>
       </c>
       <c r="I461" s="8" t="n">
-        <v>0.0352</v>
-      </c>
-      <c r="J461" s="6" t="inlineStr"/>
+        <v>0.1536</v>
+      </c>
+      <c r="J461" s="8" t="n">
+        <v>-0.1008</v>
+      </c>
       <c r="K461" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L461" s="6" t="inlineStr"/>
+          <t>Teknoloji hizmetleri</t>
+        </is>
+      </c>
+      <c r="L461" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST YILDIZ, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST SÜRDÜRÜLEBİLİRLİK, BIST KURUMSAL YÖNETİM</t>
+        </is>
+      </c>
       <c r="M461" s="6" t="inlineStr"/>
     </row>
     <row r="462">
       <c r="A462" s="2" t="inlineStr">
         <is>
-          <t>BALSU</t>
+          <t>SUMAS</t>
         </is>
       </c>
       <c r="B462" s="3" t="n">
-        <v>14.4</v>
+        <v>349.25</v>
       </c>
       <c r="C462" s="4" t="n">
-        <v>-0.0083</v>
+        <v>0.1</v>
       </c>
       <c r="D462" s="5" t="n">
-        <v>7510000</v>
+        <v>8880</v>
       </c>
       <c r="E462" s="4" t="n">
-        <v>0.25</v>
+        <v>0.3229</v>
       </c>
       <c r="F462" s="3" t="n">
-        <v>43.31</v>
-      </c>
-      <c r="G462" s="2" t="inlineStr"/>
+        <v>81.84999999999999</v>
+      </c>
+      <c r="G462" s="3" t="n">
+        <v>135.22</v>
+      </c>
       <c r="H462" s="3" t="n">
-        <v>4.38</v>
-      </c>
-      <c r="I462" s="2" t="inlineStr"/>
-      <c r="J462" s="4" t="n">
-        <v>0.9449</v>
-      </c>
+        <v>4.31</v>
+      </c>
+      <c r="I462" s="4" t="n">
+        <v>0.0352</v>
+      </c>
+      <c r="J462" s="2" t="inlineStr"/>
       <c r="K462" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
-        </is>
-      </c>
-      <c r="L462" s="2" t="inlineStr">
-        <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST GIDA ICECEK, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST 100-30, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L462" s="2" t="inlineStr"/>
       <c r="M462" s="2" t="inlineStr"/>
     </row>
     <row r="463">
       <c r="A463" s="6" t="inlineStr">
         <is>
-          <t>ALCAR</t>
+          <t>BALSU</t>
         </is>
       </c>
       <c r="B463" s="7" t="n">
-        <v>768</v>
+        <v>14.4</v>
       </c>
       <c r="C463" s="8" t="n">
-        <v>-0.0097</v>
+        <v>-0.0083</v>
       </c>
       <c r="D463" s="9" t="n">
-        <v>33640</v>
+        <v>7510000</v>
       </c>
       <c r="E463" s="8" t="n">
-        <v>0.1594</v>
+        <v>0.25</v>
       </c>
       <c r="F463" s="7" t="n">
-        <v>47.71</v>
+        <v>43.31</v>
       </c>
       <c r="G463" s="6" t="inlineStr"/>
       <c r="H463" s="7" t="n">
         <v>4.38</v>
       </c>
-      <c r="I463" s="8" t="n">
-        <v>-0.292</v>
-      </c>
+      <c r="I463" s="6" t="inlineStr"/>
       <c r="J463" s="8" t="n">
-        <v>-3.2624</v>
+        <v>0.9449</v>
       </c>
       <c r="K463" s="6" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L463" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST METAL ESYA MAKİNA, BIST İSTANBUL, BIST ANA</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST GIDA ICECEK, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST 100-30, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M463" s="6" t="inlineStr"/>
@@ -20662,42 +20660,42 @@
     <row r="464">
       <c r="A464" s="2" t="inlineStr">
         <is>
-          <t>AYCES</t>
+          <t>ALCAR</t>
         </is>
       </c>
       <c r="B464" s="3" t="n">
-        <v>853.5</v>
+        <v>768</v>
       </c>
       <c r="C464" s="4" t="n">
-        <v>-0.09970000000000001</v>
+        <v>-0.0097</v>
       </c>
       <c r="D464" s="5" t="n">
-        <v>121650</v>
+        <v>33640</v>
       </c>
       <c r="E464" s="4" t="n">
-        <v>0.0814</v>
+        <v>0.1594</v>
       </c>
       <c r="F464" s="3" t="n">
-        <v>33.91</v>
+        <v>47.71</v>
       </c>
       <c r="G464" s="2" t="inlineStr"/>
       <c r="H464" s="3" t="n">
-        <v>4.45</v>
+        <v>4.38</v>
       </c>
       <c r="I464" s="4" t="n">
-        <v>-0.016</v>
+        <v>-0.292</v>
       </c>
       <c r="J464" s="4" t="n">
-        <v>-2.6951</v>
+        <v>-3.2624</v>
       </c>
       <c r="K464" s="2" t="inlineStr">
         <is>
-          <t>Tüketici hizmetleri</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L464" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TURİZM, BIST HİZMETLER, BIST ANA, BIST İZMİR</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST METAL ESYA MAKİNA, BIST İSTANBUL, BIST ANA</t>
         </is>
       </c>
       <c r="M464" s="2" t="inlineStr"/>
@@ -20705,42 +20703,42 @@
     <row r="465">
       <c r="A465" s="6" t="inlineStr">
         <is>
-          <t>FZLGY</t>
+          <t>AYCES</t>
         </is>
       </c>
       <c r="B465" s="7" t="n">
-        <v>14.6</v>
+        <v>853.5</v>
       </c>
       <c r="C465" s="8" t="n">
-        <v>-0.004099999999999999</v>
+        <v>-0.09970000000000001</v>
       </c>
       <c r="D465" s="9" t="n">
-        <v>17090000</v>
+        <v>121650</v>
       </c>
       <c r="E465" s="8" t="n">
-        <v>0.3987</v>
+        <v>0.0814</v>
       </c>
       <c r="F465" s="7" t="n">
-        <v>43.17</v>
+        <v>33.91</v>
       </c>
       <c r="G465" s="6" t="inlineStr"/>
       <c r="H465" s="7" t="n">
-        <v>4.46</v>
+        <v>4.45</v>
       </c>
       <c r="I465" s="8" t="n">
-        <v>-0.1177</v>
+        <v>-0.016</v>
       </c>
       <c r="J465" s="8" t="n">
-        <v>-14.5611</v>
+        <v>-2.6951</v>
       </c>
       <c r="K465" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı tüketim malları</t>
+          <t>Tüketici hizmetleri</t>
         </is>
       </c>
       <c r="L465" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TURİZM, BIST HİZMETLER, BIST ANA, BIST İZMİR</t>
         </is>
       </c>
       <c r="M465" s="6" t="inlineStr"/>
@@ -20748,44 +20746,42 @@
     <row r="466">
       <c r="A466" s="2" t="inlineStr">
         <is>
-          <t>PSDTC</t>
+          <t>FZLGY</t>
         </is>
       </c>
       <c r="B466" s="3" t="n">
-        <v>134.5</v>
+        <v>14.6</v>
       </c>
       <c r="C466" s="4" t="n">
-        <v>0.0015</v>
+        <v>-0.004099999999999999</v>
       </c>
       <c r="D466" s="5" t="n">
-        <v>66170</v>
+        <v>17090000</v>
       </c>
       <c r="E466" s="4" t="n">
-        <v>0.5889</v>
+        <v>0.3987</v>
       </c>
       <c r="F466" s="3" t="n">
-        <v>52.41</v>
-      </c>
-      <c r="G466" s="3" t="n">
-        <v>19.13</v>
-      </c>
+        <v>43.17</v>
+      </c>
+      <c r="G466" s="2" t="inlineStr"/>
       <c r="H466" s="3" t="n">
-        <v>4.5</v>
+        <v>4.46</v>
       </c>
       <c r="I466" s="4" t="n">
-        <v>0.2892</v>
+        <v>-0.1177</v>
       </c>
       <c r="J466" s="4" t="n">
-        <v>0.2476</v>
+        <v>-14.5611</v>
       </c>
       <c r="K466" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Dayanıklı tüketim malları</t>
         </is>
       </c>
       <c r="L466" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İZMİR</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M466" s="2" t="inlineStr"/>
@@ -20793,42 +20789,44 @@
     <row r="467">
       <c r="A467" s="6" t="inlineStr">
         <is>
-          <t>INVES</t>
+          <t>PSDTC</t>
         </is>
       </c>
       <c r="B467" s="7" t="n">
-        <v>566</v>
+        <v>134.5</v>
       </c>
       <c r="C467" s="8" t="n">
-        <v>0.0089</v>
+        <v>0.0015</v>
       </c>
       <c r="D467" s="9" t="n">
-        <v>149300</v>
+        <v>66170</v>
       </c>
       <c r="E467" s="8" t="n">
-        <v>0.2</v>
+        <v>0.5889</v>
       </c>
       <c r="F467" s="7" t="n">
-        <v>67.09999999999999</v>
-      </c>
-      <c r="G467" s="6" t="inlineStr"/>
+        <v>52.41</v>
+      </c>
+      <c r="G467" s="7" t="n">
+        <v>19.13</v>
+      </c>
       <c r="H467" s="7" t="n">
-        <v>4.51</v>
+        <v>4.5</v>
       </c>
       <c r="I467" s="8" t="n">
-        <v>-0.0941</v>
+        <v>0.2892</v>
       </c>
       <c r="J467" s="8" t="n">
-        <v>-1.7771</v>
+        <v>0.2476</v>
       </c>
       <c r="K467" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L467" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST İSTANBUL, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İZMİR</t>
         </is>
       </c>
       <c r="M467" s="6" t="inlineStr"/>
@@ -20836,42 +20834,42 @@
     <row r="468">
       <c r="A468" s="2" t="inlineStr">
         <is>
-          <t>ARFYE</t>
+          <t>INVES</t>
         </is>
       </c>
       <c r="B468" s="3" t="n">
-        <v>33.04</v>
+        <v>566</v>
       </c>
       <c r="C468" s="4" t="n">
-        <v>0.0018</v>
+        <v>0.0089</v>
       </c>
       <c r="D468" s="5" t="n">
-        <v>10660000</v>
+        <v>149300</v>
       </c>
       <c r="E468" s="4" t="n">
-        <v>0.2571</v>
+        <v>0.2</v>
       </c>
       <c r="F468" s="3" t="n">
-        <v>62.8</v>
+        <v>67.09999999999999</v>
       </c>
       <c r="G468" s="2" t="inlineStr"/>
       <c r="H468" s="3" t="n">
-        <v>4.52</v>
+        <v>4.51</v>
       </c>
       <c r="I468" s="4" t="n">
-        <v>-0.0955</v>
+        <v>-0.0941</v>
       </c>
       <c r="J468" s="4" t="n">
-        <v>-0.2029</v>
+        <v>-1.7771</v>
       </c>
       <c r="K468" s="2" t="inlineStr">
         <is>
-          <t>Elektrik, Su, Gaz Hizmetleri</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L468" s="2" t="inlineStr">
         <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST KATILIM TÜM, BIST ANA, BIST İZMİR</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST İSTANBUL, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M468" s="2" t="inlineStr"/>
@@ -25963,23 +25961,21 @@
     <row r="587">
       <c r="A587" s="6" t="inlineStr">
         <is>
-          <t>INTEK</t>
+          <t>ENPRA</t>
         </is>
       </c>
       <c r="B587" s="7" t="n">
-        <v>240.1</v>
+        <v>82.09999999999999</v>
       </c>
       <c r="C587" s="8" t="n">
-        <v>-0.0008</v>
-      </c>
-      <c r="D587" s="7" t="n">
-        <v>8029.999999999999</v>
-      </c>
-      <c r="E587" s="8" t="n">
-        <v>0.2578</v>
-      </c>
+        <v>-0.0453</v>
+      </c>
+      <c r="D587" s="9" t="n">
+        <v>210450</v>
+      </c>
+      <c r="E587" s="6" t="inlineStr"/>
       <c r="F587" s="7" t="n">
-        <v>40.66</v>
+        <v>10.5</v>
       </c>
       <c r="G587" s="6" t="inlineStr"/>
       <c r="H587" s="6" t="inlineStr"/>
@@ -25987,7 +25983,7 @@
       <c r="J587" s="6" t="inlineStr"/>
       <c r="K587" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L587" s="6" t="inlineStr"/>
@@ -25996,34 +25992,40 @@
     <row r="588">
       <c r="A588" s="2" t="inlineStr">
         <is>
-          <t>SMRVA</t>
+          <t>ARZUM</t>
         </is>
       </c>
       <c r="B588" s="3" t="n">
-        <v>19.36</v>
+        <v>2.63</v>
       </c>
       <c r="C588" s="4" t="n">
-        <v>-0.0759</v>
+        <v>-0.0223</v>
       </c>
       <c r="D588" s="5" t="n">
-        <v>84430000</v>
-      </c>
-      <c r="E588" s="2" t="inlineStr"/>
+        <v>54820000</v>
+      </c>
+      <c r="E588" s="4" t="n">
+        <v>0.7119</v>
+      </c>
       <c r="F588" s="3" t="n">
-        <v>59.13</v>
+        <v>40.78</v>
       </c>
       <c r="G588" s="2" t="inlineStr"/>
       <c r="H588" s="2" t="inlineStr"/>
-      <c r="I588" s="2" t="inlineStr"/>
-      <c r="J588" s="2" t="inlineStr"/>
+      <c r="I588" s="4" t="n">
+        <v>-191.6342</v>
+      </c>
+      <c r="J588" s="4" t="n">
+        <v>-0.8093</v>
+      </c>
       <c r="K588" s="2" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>Dağıtım servisleri</t>
         </is>
       </c>
       <c r="L588" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M588" s="2" t="inlineStr"/>
@@ -26031,32 +26033,26 @@
     <row r="589">
       <c r="A589" s="6" t="inlineStr">
         <is>
-          <t>GRNYO</t>
+          <t>MARMR</t>
         </is>
       </c>
       <c r="B589" s="7" t="n">
-        <v>18.54</v>
+        <v>2.83</v>
       </c>
       <c r="C589" s="8" t="n">
-        <v>0.0226</v>
+        <v>-0.0174</v>
       </c>
       <c r="D589" s="9" t="n">
-        <v>1030000</v>
-      </c>
-      <c r="E589" s="8" t="n">
-        <v>0.9869</v>
-      </c>
+        <v>210300000</v>
+      </c>
+      <c r="E589" s="6" t="inlineStr"/>
       <c r="F589" s="7" t="n">
-        <v>61.23</v>
+        <v>51.51</v>
       </c>
       <c r="G589" s="6" t="inlineStr"/>
       <c r="H589" s="6" t="inlineStr"/>
-      <c r="I589" s="8" t="n">
-        <v>-0.2446</v>
-      </c>
-      <c r="J589" s="8" t="n">
-        <v>0.3246</v>
-      </c>
+      <c r="I589" s="6" t="inlineStr"/>
+      <c r="J589" s="6" t="inlineStr"/>
       <c r="K589" s="6" t="inlineStr">
         <is>
           <t>Finans</t>
@@ -26064,7 +26060,7 @@
       </c>
       <c r="L589" s="6" t="inlineStr">
         <is>
-          <t>BIST MENKUL KIYM YO</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M589" s="6" t="inlineStr"/>
@@ -26072,21 +26068,21 @@
     <row r="590">
       <c r="A590" s="2" t="inlineStr">
         <is>
-          <t>GENKM</t>
+          <t>GLRMK</t>
         </is>
       </c>
       <c r="B590" s="3" t="n">
-        <v>14.46</v>
+        <v>191</v>
       </c>
       <c r="C590" s="4" t="n">
-        <v>0.0255</v>
+        <v>0.0053</v>
       </c>
       <c r="D590" s="5" t="n">
-        <v>31020000</v>
+        <v>18010000</v>
       </c>
       <c r="E590" s="2" t="inlineStr"/>
       <c r="F590" s="3" t="n">
-        <v>58.72</v>
+        <v>45.76</v>
       </c>
       <c r="G590" s="2" t="inlineStr"/>
       <c r="H590" s="2" t="inlineStr"/>
@@ -26094,12 +26090,12 @@
       <c r="J590" s="2" t="inlineStr"/>
       <c r="K590" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L590" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
         </is>
       </c>
       <c r="M590" s="2" t="inlineStr"/>
@@ -26107,21 +26103,21 @@
     <row r="591">
       <c r="A591" s="6" t="inlineStr">
         <is>
-          <t>GLRMK</t>
+          <t>GENKM</t>
         </is>
       </c>
       <c r="B591" s="7" t="n">
-        <v>191</v>
+        <v>14.46</v>
       </c>
       <c r="C591" s="8" t="n">
-        <v>0.0053</v>
+        <v>0.0255</v>
       </c>
       <c r="D591" s="9" t="n">
-        <v>18010000</v>
+        <v>31020000</v>
       </c>
       <c r="E591" s="6" t="inlineStr"/>
       <c r="F591" s="7" t="n">
-        <v>45.76</v>
+        <v>58.72</v>
       </c>
       <c r="G591" s="6" t="inlineStr"/>
       <c r="H591" s="6" t="inlineStr"/>
@@ -26129,12 +26125,12 @@
       <c r="J591" s="6" t="inlineStr"/>
       <c r="K591" s="6" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L591" s="6" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M591" s="6" t="inlineStr"/>
@@ -26142,21 +26138,23 @@
     <row r="592">
       <c r="A592" s="2" t="inlineStr">
         <is>
-          <t>BESTE</t>
+          <t>ICUGS</t>
         </is>
       </c>
       <c r="B592" s="3" t="n">
-        <v>29.22</v>
+        <v>6.07</v>
       </c>
       <c r="C592" s="4" t="n">
-        <v>-0.0214</v>
+        <v>-0.0272</v>
       </c>
       <c r="D592" s="5" t="n">
-        <v>22260000</v>
-      </c>
-      <c r="E592" s="2" t="inlineStr"/>
+        <v>58970000</v>
+      </c>
+      <c r="E592" s="4" t="n">
+        <v>0.8667</v>
+      </c>
       <c r="F592" s="3" t="n">
-        <v>67.41</v>
+        <v>82.51000000000001</v>
       </c>
       <c r="G592" s="2" t="inlineStr"/>
       <c r="H592" s="2" t="inlineStr"/>
@@ -26164,12 +26162,12 @@
       <c r="J592" s="2" t="inlineStr"/>
       <c r="K592" s="2" t="inlineStr">
         <is>
-          <t>Elektrik, Su, Gaz Hizmetleri</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L592" s="2" t="inlineStr">
         <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
         </is>
       </c>
       <c r="M592" s="2" t="inlineStr"/>
@@ -26177,21 +26175,21 @@
     <row r="593">
       <c r="A593" s="6" t="inlineStr">
         <is>
-          <t>AAGYO</t>
+          <t>DMLKT</t>
         </is>
       </c>
       <c r="B593" s="7" t="n">
-        <v>18.37</v>
+        <v>6.15</v>
       </c>
       <c r="C593" s="8" t="n">
-        <v>-0.0113</v>
+        <v>-0.0032</v>
       </c>
       <c r="D593" s="9" t="n">
-        <v>50560000</v>
+        <v>6880000</v>
       </c>
       <c r="E593" s="6" t="inlineStr"/>
       <c r="F593" s="7" t="n">
-        <v>27.15</v>
+        <v>60.46</v>
       </c>
       <c r="G593" s="6" t="inlineStr"/>
       <c r="H593" s="6" t="inlineStr"/>
@@ -26202,95 +26200,105 @@
           <t>Finans</t>
         </is>
       </c>
-      <c r="L593" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
-        </is>
-      </c>
+      <c r="L593" s="6" t="inlineStr"/>
       <c r="M593" s="6" t="inlineStr"/>
     </row>
     <row r="594">
       <c r="A594" s="2" t="inlineStr">
         <is>
-          <t>ALTIN</t>
+          <t>MMCAS</t>
         </is>
       </c>
       <c r="B594" s="3" t="n">
-        <v>79.78</v>
+        <v>81.2</v>
       </c>
       <c r="C594" s="4" t="n">
-        <v>0.0036</v>
+        <v>-0.05690000000000001</v>
       </c>
       <c r="D594" s="5" t="n">
-        <v>9710000</v>
-      </c>
-      <c r="E594" s="2" t="inlineStr"/>
+        <v>48270</v>
+      </c>
+      <c r="E594" s="4" t="n">
+        <v>0.58</v>
+      </c>
       <c r="F594" s="3" t="n">
-        <v>41.39</v>
+        <v>47.53</v>
       </c>
       <c r="G594" s="2" t="inlineStr"/>
       <c r="H594" s="2" t="inlineStr"/>
-      <c r="I594" s="2" t="inlineStr"/>
-      <c r="J594" s="2" t="inlineStr"/>
-      <c r="K594" s="2" t="inlineStr"/>
+      <c r="I594" s="4" t="n">
+        <v>-9.409700000000001</v>
+      </c>
+      <c r="J594" s="4" t="n">
+        <v>-4.155</v>
+      </c>
+      <c r="K594" s="2" t="inlineStr">
+        <is>
+          <t>Taşımacılık</t>
+        </is>
+      </c>
       <c r="L594" s="2" t="inlineStr"/>
       <c r="M594" s="2" t="inlineStr"/>
     </row>
     <row r="595">
       <c r="A595" s="6" t="inlineStr">
         <is>
-          <t>BRMEN</t>
+          <t>GRNYO</t>
         </is>
       </c>
       <c r="B595" s="7" t="n">
-        <v>6.75</v>
+        <v>18.54</v>
       </c>
       <c r="C595" s="8" t="n">
-        <v>0.0433</v>
+        <v>0.0226</v>
       </c>
       <c r="D595" s="9" t="n">
-        <v>707270</v>
+        <v>1030000</v>
       </c>
       <c r="E595" s="8" t="n">
-        <v>0.95</v>
+        <v>0.9869</v>
       </c>
       <c r="F595" s="7" t="n">
-        <v>37.16</v>
+        <v>61.23</v>
       </c>
       <c r="G595" s="6" t="inlineStr"/>
       <c r="H595" s="6" t="inlineStr"/>
       <c r="I595" s="8" t="n">
-        <v>-23.6291</v>
+        <v>-0.2446</v>
       </c>
       <c r="J595" s="8" t="n">
-        <v>-0.4678</v>
+        <v>0.3246</v>
       </c>
       <c r="K595" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L595" s="6" t="inlineStr"/>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L595" s="6" t="inlineStr">
+        <is>
+          <t>BIST MENKUL KIYM YO</t>
+        </is>
+      </c>
       <c r="M595" s="6" t="inlineStr"/>
     </row>
     <row r="596">
       <c r="A596" s="2" t="inlineStr">
         <is>
-          <t>DMLKT</t>
+          <t>CGCAM</t>
         </is>
       </c>
       <c r="B596" s="3" t="n">
-        <v>6.15</v>
+        <v>42.14</v>
       </c>
       <c r="C596" s="4" t="n">
-        <v>-0.0032</v>
+        <v>0.0354</v>
       </c>
       <c r="D596" s="5" t="n">
-        <v>6880000</v>
+        <v>6400000</v>
       </c>
       <c r="E596" s="2" t="inlineStr"/>
       <c r="F596" s="3" t="n">
-        <v>60.46</v>
+        <v>59.11</v>
       </c>
       <c r="G596" s="2" t="inlineStr"/>
       <c r="H596" s="2" t="inlineStr"/>
@@ -26298,30 +26306,34 @@
       <c r="J596" s="2" t="inlineStr"/>
       <c r="K596" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L596" s="2" t="inlineStr"/>
+          <t>Dayanıklı tüketim malları</t>
+        </is>
+      </c>
+      <c r="L596" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
+        </is>
+      </c>
       <c r="M596" s="2" t="inlineStr"/>
     </row>
     <row r="597">
       <c r="A597" s="6" t="inlineStr">
         <is>
-          <t>EMPAE</t>
+          <t>FRMPL</t>
         </is>
       </c>
       <c r="B597" s="7" t="n">
-        <v>42.98</v>
+        <v>33.98</v>
       </c>
       <c r="C597" s="8" t="n">
-        <v>0.0998</v>
-      </c>
-      <c r="D597" s="9" t="n">
-        <v>11900000</v>
+        <v>0.0253</v>
+      </c>
+      <c r="D597" s="7" t="n">
+        <v>4020000</v>
       </c>
       <c r="E597" s="6" t="inlineStr"/>
       <c r="F597" s="7" t="n">
-        <v>59.61</v>
+        <v>53.84</v>
       </c>
       <c r="G597" s="6" t="inlineStr"/>
       <c r="H597" s="6" t="inlineStr"/>
@@ -26329,12 +26341,12 @@
       <c r="J597" s="6" t="inlineStr"/>
       <c r="K597" s="6" t="inlineStr">
         <is>
-          <t>Elektronik teknoloji</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L597" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M597" s="6" t="inlineStr"/>
@@ -26342,36 +26354,38 @@
     <row r="598">
       <c r="A598" s="2" t="inlineStr">
         <is>
-          <t>ICUGS</t>
+          <t>NETAS</t>
         </is>
       </c>
       <c r="B598" s="3" t="n">
-        <v>6.07</v>
+        <v>67.45</v>
       </c>
       <c r="C598" s="4" t="n">
-        <v>-0.0272</v>
+        <v>0.0622</v>
       </c>
       <c r="D598" s="5" t="n">
-        <v>58970000</v>
+        <v>798460</v>
       </c>
       <c r="E598" s="4" t="n">
-        <v>0.8667</v>
+        <v>0.3695000000000001</v>
       </c>
       <c r="F598" s="3" t="n">
-        <v>82.51000000000001</v>
+        <v>61.76</v>
       </c>
       <c r="G598" s="2" t="inlineStr"/>
       <c r="H598" s="2" t="inlineStr"/>
       <c r="I598" s="2" t="inlineStr"/>
-      <c r="J598" s="2" t="inlineStr"/>
+      <c r="J598" s="4" t="n">
+        <v>0.4139</v>
+      </c>
       <c r="K598" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Teknoloji hizmetleri</t>
         </is>
       </c>
       <c r="L598" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M598" s="2" t="inlineStr"/>
@@ -26379,21 +26393,21 @@
     <row r="599">
       <c r="A599" s="6" t="inlineStr">
         <is>
-          <t>MARMR</t>
+          <t>SMRVA</t>
         </is>
       </c>
       <c r="B599" s="7" t="n">
-        <v>2.83</v>
+        <v>19.36</v>
       </c>
       <c r="C599" s="8" t="n">
-        <v>-0.0174</v>
+        <v>-0.0759</v>
       </c>
       <c r="D599" s="9" t="n">
-        <v>210300000</v>
+        <v>84430000</v>
       </c>
       <c r="E599" s="6" t="inlineStr"/>
       <c r="F599" s="7" t="n">
-        <v>51.51</v>
+        <v>59.13</v>
       </c>
       <c r="G599" s="6" t="inlineStr"/>
       <c r="H599" s="6" t="inlineStr"/>
@@ -26401,12 +26415,12 @@
       <c r="J599" s="6" t="inlineStr"/>
       <c r="K599" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L599" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
         </is>
       </c>
       <c r="M599" s="6" t="inlineStr"/>
@@ -26414,40 +26428,34 @@
     <row r="600">
       <c r="A600" s="2" t="inlineStr">
         <is>
-          <t>BORLS</t>
+          <t>EMPAE</t>
         </is>
       </c>
       <c r="B600" s="3" t="n">
-        <v>8.81</v>
+        <v>42.98</v>
       </c>
       <c r="C600" s="4" t="n">
-        <v>0.0513</v>
+        <v>0.0998</v>
       </c>
       <c r="D600" s="5" t="n">
-        <v>106140000</v>
-      </c>
-      <c r="E600" s="4" t="n">
-        <v>0.1672</v>
-      </c>
+        <v>11900000</v>
+      </c>
+      <c r="E600" s="2" t="inlineStr"/>
       <c r="F600" s="3" t="n">
-        <v>75.73</v>
+        <v>59.61</v>
       </c>
       <c r="G600" s="2" t="inlineStr"/>
       <c r="H600" s="2" t="inlineStr"/>
-      <c r="I600" s="4" t="n">
-        <v>-5.3262</v>
-      </c>
-      <c r="J600" s="4" t="n">
-        <v>-4.2562</v>
-      </c>
+      <c r="I600" s="2" t="inlineStr"/>
+      <c r="J600" s="2" t="inlineStr"/>
       <c r="K600" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Elektronik teknoloji</t>
         </is>
       </c>
       <c r="L600" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
         </is>
       </c>
       <c r="M600" s="2" t="inlineStr"/>
@@ -26455,42 +26463,34 @@
     <row r="601">
       <c r="A601" s="6" t="inlineStr">
         <is>
-          <t>BERA</t>
+          <t>AAGYO</t>
         </is>
       </c>
       <c r="B601" s="7" t="n">
-        <v>17.35</v>
+        <v>18.37</v>
       </c>
       <c r="C601" s="8" t="n">
-        <v>0.014</v>
+        <v>-0.0113</v>
       </c>
       <c r="D601" s="9" t="n">
-        <v>11300000</v>
-      </c>
-      <c r="E601" s="8" t="n">
-        <v>0.9246</v>
-      </c>
+        <v>50560000</v>
+      </c>
+      <c r="E601" s="6" t="inlineStr"/>
       <c r="F601" s="7" t="n">
-        <v>50.67</v>
-      </c>
-      <c r="G601" s="7" t="n">
-        <v>163.99</v>
-      </c>
+        <v>27.15</v>
+      </c>
+      <c r="G601" s="6" t="inlineStr"/>
       <c r="H601" s="6" t="inlineStr"/>
-      <c r="I601" s="8" t="n">
-        <v>0.0028</v>
-      </c>
-      <c r="J601" s="8" t="n">
-        <v>-10.3171</v>
-      </c>
+      <c r="I601" s="6" t="inlineStr"/>
+      <c r="J601" s="6" t="inlineStr"/>
       <c r="K601" s="6" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L601" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KONYA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M601" s="6" t="inlineStr"/>
@@ -26498,21 +26498,23 @@
     <row r="602">
       <c r="A602" s="2" t="inlineStr">
         <is>
-          <t>MCARD</t>
+          <t>INTEK</t>
         </is>
       </c>
       <c r="B602" s="3" t="n">
-        <v>178.6</v>
+        <v>240.1</v>
       </c>
       <c r="C602" s="4" t="n">
-        <v>0.0998</v>
-      </c>
-      <c r="D602" s="5" t="n">
-        <v>6520000</v>
-      </c>
-      <c r="E602" s="2" t="inlineStr"/>
+        <v>-0.0008</v>
+      </c>
+      <c r="D602" s="3" t="n">
+        <v>8029.999999999999</v>
+      </c>
+      <c r="E602" s="4" t="n">
+        <v>0.2578</v>
+      </c>
       <c r="F602" s="3" t="n">
-        <v>62.69</v>
+        <v>40.66</v>
       </c>
       <c r="G602" s="2" t="inlineStr"/>
       <c r="H602" s="2" t="inlineStr"/>
@@ -26520,53 +26522,49 @@
       <c r="J602" s="2" t="inlineStr"/>
       <c r="K602" s="2" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
-        </is>
-      </c>
-      <c r="L602" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L602" s="2" t="inlineStr"/>
       <c r="M602" s="2" t="inlineStr"/>
     </row>
     <row r="603">
       <c r="A603" s="6" t="inlineStr">
         <is>
-          <t>CRFSA</t>
+          <t>BORLS</t>
         </is>
       </c>
       <c r="B603" s="7" t="n">
-        <v>147</v>
+        <v>8.81</v>
       </c>
       <c r="C603" s="8" t="n">
-        <v>0.0138</v>
+        <v>0.0513</v>
       </c>
       <c r="D603" s="9" t="n">
-        <v>2130000</v>
+        <v>106140000</v>
       </c>
       <c r="E603" s="8" t="n">
-        <v>0.1071</v>
+        <v>0.1672</v>
       </c>
       <c r="F603" s="7" t="n">
-        <v>50.74</v>
+        <v>75.73</v>
       </c>
       <c r="G603" s="6" t="inlineStr"/>
       <c r="H603" s="6" t="inlineStr"/>
       <c r="I603" s="8" t="n">
-        <v>-3.6635</v>
+        <v>-5.3262</v>
       </c>
       <c r="J603" s="8" t="n">
-        <v>-0.4897</v>
+        <v>-4.2562</v>
       </c>
       <c r="K603" s="6" t="inlineStr">
         <is>
-          <t>Perakende satış</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L603" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M603" s="6" t="inlineStr"/>
@@ -26574,40 +26572,34 @@
     <row r="604">
       <c r="A604" s="2" t="inlineStr">
         <is>
-          <t>ARZUM</t>
+          <t>BESTE</t>
         </is>
       </c>
       <c r="B604" s="3" t="n">
-        <v>2.63</v>
+        <v>29.22</v>
       </c>
       <c r="C604" s="4" t="n">
-        <v>-0.0223</v>
+        <v>-0.0214</v>
       </c>
       <c r="D604" s="5" t="n">
-        <v>54820000</v>
-      </c>
-      <c r="E604" s="4" t="n">
-        <v>0.7119</v>
-      </c>
+        <v>22260000</v>
+      </c>
+      <c r="E604" s="2" t="inlineStr"/>
       <c r="F604" s="3" t="n">
-        <v>40.78</v>
+        <v>67.41</v>
       </c>
       <c r="G604" s="2" t="inlineStr"/>
       <c r="H604" s="2" t="inlineStr"/>
-      <c r="I604" s="4" t="n">
-        <v>-191.6342</v>
-      </c>
-      <c r="J604" s="4" t="n">
-        <v>-0.8093</v>
-      </c>
+      <c r="I604" s="2" t="inlineStr"/>
+      <c r="J604" s="2" t="inlineStr"/>
       <c r="K604" s="2" t="inlineStr">
         <is>
-          <t>Dağıtım servisleri</t>
+          <t>Elektrik, Su, Gaz Hizmetleri</t>
         </is>
       </c>
       <c r="L604" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M604" s="2" t="inlineStr"/>
@@ -26615,75 +26607,69 @@
     <row r="605">
       <c r="A605" s="6" t="inlineStr">
         <is>
-          <t>MMCAS</t>
+          <t>ALTIN</t>
         </is>
       </c>
       <c r="B605" s="7" t="n">
-        <v>81.2</v>
+        <v>79.78</v>
       </c>
       <c r="C605" s="8" t="n">
-        <v>-0.05690000000000001</v>
+        <v>0.0036</v>
       </c>
       <c r="D605" s="9" t="n">
-        <v>48270</v>
-      </c>
-      <c r="E605" s="8" t="n">
-        <v>0.58</v>
-      </c>
+        <v>9710000</v>
+      </c>
+      <c r="E605" s="6" t="inlineStr"/>
       <c r="F605" s="7" t="n">
-        <v>47.53</v>
+        <v>41.39</v>
       </c>
       <c r="G605" s="6" t="inlineStr"/>
       <c r="H605" s="6" t="inlineStr"/>
-      <c r="I605" s="8" t="n">
-        <v>-9.409700000000001</v>
-      </c>
-      <c r="J605" s="8" t="n">
-        <v>-4.155</v>
-      </c>
-      <c r="K605" s="6" t="inlineStr">
-        <is>
-          <t>Taşımacılık</t>
-        </is>
-      </c>
+      <c r="I605" s="6" t="inlineStr"/>
+      <c r="J605" s="6" t="inlineStr"/>
+      <c r="K605" s="6" t="inlineStr"/>
       <c r="L605" s="6" t="inlineStr"/>
       <c r="M605" s="6" t="inlineStr"/>
     </row>
     <row r="606">
       <c r="A606" s="2" t="inlineStr">
         <is>
-          <t>NETAS</t>
+          <t>BERA</t>
         </is>
       </c>
       <c r="B606" s="3" t="n">
-        <v>67.45</v>
+        <v>17.35</v>
       </c>
       <c r="C606" s="4" t="n">
-        <v>0.0622</v>
+        <v>0.014</v>
       </c>
       <c r="D606" s="5" t="n">
-        <v>798460</v>
+        <v>11300000</v>
       </c>
       <c r="E606" s="4" t="n">
-        <v>0.3695000000000001</v>
+        <v>0.9246</v>
       </c>
       <c r="F606" s="3" t="n">
-        <v>61.76</v>
-      </c>
-      <c r="G606" s="2" t="inlineStr"/>
+        <v>50.67</v>
+      </c>
+      <c r="G606" s="3" t="n">
+        <v>163.99</v>
+      </c>
       <c r="H606" s="2" t="inlineStr"/>
-      <c r="I606" s="2" t="inlineStr"/>
+      <c r="I606" s="4" t="n">
+        <v>0.0028</v>
+      </c>
       <c r="J606" s="4" t="n">
-        <v>0.4139</v>
+        <v>-10.3171</v>
       </c>
       <c r="K606" s="2" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L606" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KONYA</t>
         </is>
       </c>
       <c r="M606" s="2" t="inlineStr"/>
@@ -26728,21 +26714,21 @@
     <row r="608">
       <c r="A608" s="2" t="inlineStr">
         <is>
-          <t>FRMPL</t>
+          <t>LXGYO</t>
         </is>
       </c>
       <c r="B608" s="3" t="n">
-        <v>33.98</v>
+        <v>17.89</v>
       </c>
       <c r="C608" s="4" t="n">
-        <v>0.0253</v>
+        <v>0.0371</v>
       </c>
       <c r="D608" s="3" t="n">
-        <v>4020000</v>
+        <v>66540000.00000001</v>
       </c>
       <c r="E608" s="2" t="inlineStr"/>
       <c r="F608" s="3" t="n">
-        <v>53.84</v>
+        <v>56.21</v>
       </c>
       <c r="G608" s="2" t="inlineStr"/>
       <c r="H608" s="2" t="inlineStr"/>
@@ -26750,12 +26736,12 @@
       <c r="J608" s="2" t="inlineStr"/>
       <c r="K608" s="2" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L608" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M608" s="2" t="inlineStr"/>
@@ -26763,21 +26749,21 @@
     <row r="609">
       <c r="A609" s="6" t="inlineStr">
         <is>
-          <t>LXGYO</t>
+          <t>MCARD</t>
         </is>
       </c>
       <c r="B609" s="7" t="n">
-        <v>17.89</v>
+        <v>178.6</v>
       </c>
       <c r="C609" s="8" t="n">
-        <v>0.0371</v>
-      </c>
-      <c r="D609" s="7" t="n">
-        <v>66540000.00000001</v>
+        <v>0.0998</v>
+      </c>
+      <c r="D609" s="9" t="n">
+        <v>6520000</v>
       </c>
       <c r="E609" s="6" t="inlineStr"/>
       <c r="F609" s="7" t="n">
-        <v>56.21</v>
+        <v>62.69</v>
       </c>
       <c r="G609" s="6" t="inlineStr"/>
       <c r="H609" s="6" t="inlineStr"/>
@@ -26785,12 +26771,12 @@
       <c r="J609" s="6" t="inlineStr"/>
       <c r="K609" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L609" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
         </is>
       </c>
       <c r="M609" s="6" t="inlineStr"/>
@@ -26798,34 +26784,40 @@
     <row r="610">
       <c r="A610" s="2" t="inlineStr">
         <is>
-          <t>CGCAM</t>
+          <t>CRFSA</t>
         </is>
       </c>
       <c r="B610" s="3" t="n">
-        <v>42.14</v>
+        <v>147</v>
       </c>
       <c r="C610" s="4" t="n">
-        <v>0.0354</v>
+        <v>0.0138</v>
       </c>
       <c r="D610" s="5" t="n">
-        <v>6400000</v>
-      </c>
-      <c r="E610" s="2" t="inlineStr"/>
+        <v>2130000</v>
+      </c>
+      <c r="E610" s="4" t="n">
+        <v>0.1071</v>
+      </c>
       <c r="F610" s="3" t="n">
-        <v>59.11</v>
+        <v>50.74</v>
       </c>
       <c r="G610" s="2" t="inlineStr"/>
       <c r="H610" s="2" t="inlineStr"/>
-      <c r="I610" s="2" t="inlineStr"/>
-      <c r="J610" s="2" t="inlineStr"/>
+      <c r="I610" s="4" t="n">
+        <v>-3.6635</v>
+      </c>
+      <c r="J610" s="4" t="n">
+        <v>-0.4897</v>
+      </c>
       <c r="K610" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı tüketim malları</t>
+          <t>Perakende satış</t>
         </is>
       </c>
       <c r="L610" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
         </is>
       </c>
       <c r="M610" s="2" t="inlineStr"/>
@@ -26833,29 +26825,35 @@
     <row r="611">
       <c r="A611" s="6" t="inlineStr">
         <is>
-          <t>ENPRA</t>
+          <t>BRMEN</t>
         </is>
       </c>
       <c r="B611" s="7" t="n">
-        <v>82.09999999999999</v>
+        <v>6.75</v>
       </c>
       <c r="C611" s="8" t="n">
-        <v>-0.0453</v>
+        <v>0.0433</v>
       </c>
       <c r="D611" s="9" t="n">
-        <v>210450</v>
-      </c>
-      <c r="E611" s="6" t="inlineStr"/>
+        <v>707270</v>
+      </c>
+      <c r="E611" s="8" t="n">
+        <v>0.95</v>
+      </c>
       <c r="F611" s="7" t="n">
-        <v>10.5</v>
+        <v>37.16</v>
       </c>
       <c r="G611" s="6" t="inlineStr"/>
       <c r="H611" s="6" t="inlineStr"/>
-      <c r="I611" s="6" t="inlineStr"/>
-      <c r="J611" s="6" t="inlineStr"/>
+      <c r="I611" s="8" t="n">
+        <v>-23.6291</v>
+      </c>
+      <c r="J611" s="8" t="n">
+        <v>-0.4678</v>
+      </c>
       <c r="K611" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L611" s="6" t="inlineStr"/>
@@ -26883,7 +26881,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>05.05.2026 15:30</t>
+          <t>05.05.2026 16:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 BIST Screener | 05.05.2026 17:02 | 610 hisse
</commit_message>
<xml_diff>
--- a/data/bist_screener_2026-05-05.xlsx
+++ b/data/bist_screener_2026-05-05.xlsx
@@ -25961,21 +25961,21 @@
     <row r="587">
       <c r="A587" s="6" t="inlineStr">
         <is>
-          <t>ENPRA</t>
+          <t>CGCAM</t>
         </is>
       </c>
       <c r="B587" s="7" t="n">
-        <v>82.09999999999999</v>
+        <v>42.14</v>
       </c>
       <c r="C587" s="8" t="n">
-        <v>-0.0453</v>
+        <v>0.0354</v>
       </c>
       <c r="D587" s="9" t="n">
-        <v>210450</v>
+        <v>6400000</v>
       </c>
       <c r="E587" s="6" t="inlineStr"/>
       <c r="F587" s="7" t="n">
-        <v>10.5</v>
+        <v>59.11</v>
       </c>
       <c r="G587" s="6" t="inlineStr"/>
       <c r="H587" s="6" t="inlineStr"/>
@@ -25983,49 +25983,47 @@
       <c r="J587" s="6" t="inlineStr"/>
       <c r="K587" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L587" s="6" t="inlineStr"/>
+          <t>Dayanıklı tüketim malları</t>
+        </is>
+      </c>
+      <c r="L587" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
+        </is>
+      </c>
       <c r="M587" s="6" t="inlineStr"/>
     </row>
     <row r="588">
       <c r="A588" s="2" t="inlineStr">
         <is>
-          <t>ARZUM</t>
+          <t>LXGYO</t>
         </is>
       </c>
       <c r="B588" s="3" t="n">
-        <v>2.63</v>
+        <v>17.89</v>
       </c>
       <c r="C588" s="4" t="n">
-        <v>-0.0223</v>
-      </c>
-      <c r="D588" s="5" t="n">
-        <v>54820000</v>
-      </c>
-      <c r="E588" s="4" t="n">
-        <v>0.7119</v>
-      </c>
+        <v>0.0371</v>
+      </c>
+      <c r="D588" s="3" t="n">
+        <v>66540000.00000001</v>
+      </c>
+      <c r="E588" s="2" t="inlineStr"/>
       <c r="F588" s="3" t="n">
-        <v>40.78</v>
+        <v>56.21</v>
       </c>
       <c r="G588" s="2" t="inlineStr"/>
       <c r="H588" s="2" t="inlineStr"/>
-      <c r="I588" s="4" t="n">
-        <v>-191.6342</v>
-      </c>
-      <c r="J588" s="4" t="n">
-        <v>-0.8093</v>
-      </c>
+      <c r="I588" s="2" t="inlineStr"/>
+      <c r="J588" s="2" t="inlineStr"/>
       <c r="K588" s="2" t="inlineStr">
         <is>
-          <t>Dağıtım servisleri</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L588" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M588" s="2" t="inlineStr"/>
@@ -26033,34 +26031,40 @@
     <row r="589">
       <c r="A589" s="6" t="inlineStr">
         <is>
-          <t>MARMR</t>
+          <t>ARZUM</t>
         </is>
       </c>
       <c r="B589" s="7" t="n">
-        <v>2.83</v>
+        <v>2.63</v>
       </c>
       <c r="C589" s="8" t="n">
-        <v>-0.0174</v>
+        <v>-0.0223</v>
       </c>
       <c r="D589" s="9" t="n">
-        <v>210300000</v>
-      </c>
-      <c r="E589" s="6" t="inlineStr"/>
+        <v>54820000</v>
+      </c>
+      <c r="E589" s="8" t="n">
+        <v>0.7119</v>
+      </c>
       <c r="F589" s="7" t="n">
-        <v>51.51</v>
+        <v>40.78</v>
       </c>
       <c r="G589" s="6" t="inlineStr"/>
       <c r="H589" s="6" t="inlineStr"/>
-      <c r="I589" s="6" t="inlineStr"/>
-      <c r="J589" s="6" t="inlineStr"/>
+      <c r="I589" s="8" t="n">
+        <v>-191.6342</v>
+      </c>
+      <c r="J589" s="8" t="n">
+        <v>-0.8093</v>
+      </c>
       <c r="K589" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Dağıtım servisleri</t>
         </is>
       </c>
       <c r="L589" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M589" s="6" t="inlineStr"/>
@@ -26068,21 +26072,21 @@
     <row r="590">
       <c r="A590" s="2" t="inlineStr">
         <is>
-          <t>GLRMK</t>
+          <t>GENKM</t>
         </is>
       </c>
       <c r="B590" s="3" t="n">
-        <v>191</v>
+        <v>14.46</v>
       </c>
       <c r="C590" s="4" t="n">
-        <v>0.0053</v>
+        <v>0.0255</v>
       </c>
       <c r="D590" s="5" t="n">
-        <v>18010000</v>
+        <v>31020000</v>
       </c>
       <c r="E590" s="2" t="inlineStr"/>
       <c r="F590" s="3" t="n">
-        <v>45.76</v>
+        <v>58.72</v>
       </c>
       <c r="G590" s="2" t="inlineStr"/>
       <c r="H590" s="2" t="inlineStr"/>
@@ -26090,12 +26094,12 @@
       <c r="J590" s="2" t="inlineStr"/>
       <c r="K590" s="2" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L590" s="2" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M590" s="2" t="inlineStr"/>
@@ -26103,21 +26107,21 @@
     <row r="591">
       <c r="A591" s="6" t="inlineStr">
         <is>
-          <t>GENKM</t>
+          <t>EMPAE</t>
         </is>
       </c>
       <c r="B591" s="7" t="n">
-        <v>14.46</v>
+        <v>42.98</v>
       </c>
       <c r="C591" s="8" t="n">
-        <v>0.0255</v>
+        <v>0.0998</v>
       </c>
       <c r="D591" s="9" t="n">
-        <v>31020000</v>
+        <v>11900000</v>
       </c>
       <c r="E591" s="6" t="inlineStr"/>
       <c r="F591" s="7" t="n">
-        <v>58.72</v>
+        <v>59.61</v>
       </c>
       <c r="G591" s="6" t="inlineStr"/>
       <c r="H591" s="6" t="inlineStr"/>
@@ -26125,12 +26129,12 @@
       <c r="J591" s="6" t="inlineStr"/>
       <c r="K591" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Elektronik teknoloji</t>
         </is>
       </c>
       <c r="L591" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
         </is>
       </c>
       <c r="M591" s="6" t="inlineStr"/>
@@ -26138,23 +26142,21 @@
     <row r="592">
       <c r="A592" s="2" t="inlineStr">
         <is>
-          <t>ICUGS</t>
+          <t>SMRVA</t>
         </is>
       </c>
       <c r="B592" s="3" t="n">
-        <v>6.07</v>
+        <v>19.36</v>
       </c>
       <c r="C592" s="4" t="n">
-        <v>-0.0272</v>
+        <v>-0.0759</v>
       </c>
       <c r="D592" s="5" t="n">
-        <v>58970000</v>
-      </c>
-      <c r="E592" s="4" t="n">
-        <v>0.8667</v>
-      </c>
+        <v>84430000</v>
+      </c>
+      <c r="E592" s="2" t="inlineStr"/>
       <c r="F592" s="3" t="n">
-        <v>82.51000000000001</v>
+        <v>59.13</v>
       </c>
       <c r="G592" s="2" t="inlineStr"/>
       <c r="H592" s="2" t="inlineStr"/>
@@ -26162,12 +26164,12 @@
       <c r="J592" s="2" t="inlineStr"/>
       <c r="K592" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L592" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
         </is>
       </c>
       <c r="M592" s="2" t="inlineStr"/>
@@ -26175,66 +26177,70 @@
     <row r="593">
       <c r="A593" s="6" t="inlineStr">
         <is>
-          <t>DMLKT</t>
+          <t>GRNYO</t>
         </is>
       </c>
       <c r="B593" s="7" t="n">
-        <v>6.15</v>
+        <v>18.54</v>
       </c>
       <c r="C593" s="8" t="n">
-        <v>-0.0032</v>
+        <v>0.0226</v>
       </c>
       <c r="D593" s="9" t="n">
-        <v>6880000</v>
-      </c>
-      <c r="E593" s="6" t="inlineStr"/>
+        <v>1030000</v>
+      </c>
+      <c r="E593" s="8" t="n">
+        <v>0.9869</v>
+      </c>
       <c r="F593" s="7" t="n">
-        <v>60.46</v>
+        <v>61.23</v>
       </c>
       <c r="G593" s="6" t="inlineStr"/>
       <c r="H593" s="6" t="inlineStr"/>
-      <c r="I593" s="6" t="inlineStr"/>
-      <c r="J593" s="6" t="inlineStr"/>
+      <c r="I593" s="8" t="n">
+        <v>-0.2446</v>
+      </c>
+      <c r="J593" s="8" t="n">
+        <v>0.3246</v>
+      </c>
       <c r="K593" s="6" t="inlineStr">
         <is>
           <t>Finans</t>
         </is>
       </c>
-      <c r="L593" s="6" t="inlineStr"/>
+      <c r="L593" s="6" t="inlineStr">
+        <is>
+          <t>BIST MENKUL KIYM YO</t>
+        </is>
+      </c>
       <c r="M593" s="6" t="inlineStr"/>
     </row>
     <row r="594">
       <c r="A594" s="2" t="inlineStr">
         <is>
-          <t>MMCAS</t>
+          <t>ENPRA</t>
         </is>
       </c>
       <c r="B594" s="3" t="n">
-        <v>81.2</v>
+        <v>82.09999999999999</v>
       </c>
       <c r="C594" s="4" t="n">
-        <v>-0.05690000000000001</v>
+        <v>-0.0453</v>
       </c>
       <c r="D594" s="5" t="n">
-        <v>48270</v>
-      </c>
-      <c r="E594" s="4" t="n">
-        <v>0.58</v>
-      </c>
+        <v>210450</v>
+      </c>
+      <c r="E594" s="2" t="inlineStr"/>
       <c r="F594" s="3" t="n">
-        <v>47.53</v>
+        <v>10.5</v>
       </c>
       <c r="G594" s="2" t="inlineStr"/>
       <c r="H594" s="2" t="inlineStr"/>
-      <c r="I594" s="4" t="n">
-        <v>-9.409700000000001</v>
-      </c>
-      <c r="J594" s="4" t="n">
-        <v>-4.155</v>
-      </c>
+      <c r="I594" s="2" t="inlineStr"/>
+      <c r="J594" s="2" t="inlineStr"/>
       <c r="K594" s="2" t="inlineStr">
         <is>
-          <t>Taşımacılık</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L594" s="2" t="inlineStr"/>
@@ -26243,40 +26249,42 @@
     <row r="595">
       <c r="A595" s="6" t="inlineStr">
         <is>
-          <t>GRNYO</t>
+          <t>BERA</t>
         </is>
       </c>
       <c r="B595" s="7" t="n">
-        <v>18.54</v>
+        <v>17.35</v>
       </c>
       <c r="C595" s="8" t="n">
-        <v>0.0226</v>
+        <v>0.014</v>
       </c>
       <c r="D595" s="9" t="n">
-        <v>1030000</v>
+        <v>11300000</v>
       </c>
       <c r="E595" s="8" t="n">
-        <v>0.9869</v>
+        <v>0.9246</v>
       </c>
       <c r="F595" s="7" t="n">
-        <v>61.23</v>
-      </c>
-      <c r="G595" s="6" t="inlineStr"/>
+        <v>50.67</v>
+      </c>
+      <c r="G595" s="7" t="n">
+        <v>163.99</v>
+      </c>
       <c r="H595" s="6" t="inlineStr"/>
       <c r="I595" s="8" t="n">
-        <v>-0.2446</v>
+        <v>0.0028</v>
       </c>
       <c r="J595" s="8" t="n">
-        <v>0.3246</v>
+        <v>-10.3171</v>
       </c>
       <c r="K595" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L595" s="6" t="inlineStr">
         <is>
-          <t>BIST MENKUL KIYM YO</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KONYA</t>
         </is>
       </c>
       <c r="M595" s="6" t="inlineStr"/>
@@ -26284,21 +26292,21 @@
     <row r="596">
       <c r="A596" s="2" t="inlineStr">
         <is>
-          <t>CGCAM</t>
+          <t>MCARD</t>
         </is>
       </c>
       <c r="B596" s="3" t="n">
-        <v>42.14</v>
+        <v>178.6</v>
       </c>
       <c r="C596" s="4" t="n">
-        <v>0.0354</v>
+        <v>0.0998</v>
       </c>
       <c r="D596" s="5" t="n">
-        <v>6400000</v>
+        <v>6520000</v>
       </c>
       <c r="E596" s="2" t="inlineStr"/>
       <c r="F596" s="3" t="n">
-        <v>59.11</v>
+        <v>62.69</v>
       </c>
       <c r="G596" s="2" t="inlineStr"/>
       <c r="H596" s="2" t="inlineStr"/>
@@ -26306,12 +26314,12 @@
       <c r="J596" s="2" t="inlineStr"/>
       <c r="K596" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı tüketim malları</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L596" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
         </is>
       </c>
       <c r="M596" s="2" t="inlineStr"/>
@@ -26319,36 +26327,38 @@
     <row r="597">
       <c r="A597" s="6" t="inlineStr">
         <is>
-          <t>FRMPL</t>
+          <t>MMCAS</t>
         </is>
       </c>
       <c r="B597" s="7" t="n">
-        <v>33.98</v>
+        <v>81.2</v>
       </c>
       <c r="C597" s="8" t="n">
-        <v>0.0253</v>
-      </c>
-      <c r="D597" s="7" t="n">
-        <v>4020000</v>
-      </c>
-      <c r="E597" s="6" t="inlineStr"/>
+        <v>-0.05690000000000001</v>
+      </c>
+      <c r="D597" s="9" t="n">
+        <v>48270</v>
+      </c>
+      <c r="E597" s="8" t="n">
+        <v>0.58</v>
+      </c>
       <c r="F597" s="7" t="n">
-        <v>53.84</v>
+        <v>47.53</v>
       </c>
       <c r="G597" s="6" t="inlineStr"/>
       <c r="H597" s="6" t="inlineStr"/>
-      <c r="I597" s="6" t="inlineStr"/>
-      <c r="J597" s="6" t="inlineStr"/>
+      <c r="I597" s="8" t="n">
+        <v>-9.409700000000001</v>
+      </c>
+      <c r="J597" s="8" t="n">
+        <v>-4.155</v>
+      </c>
       <c r="K597" s="6" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
-        </is>
-      </c>
-      <c r="L597" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
-        </is>
-      </c>
+          <t>Taşımacılık</t>
+        </is>
+      </c>
+      <c r="L597" s="6" t="inlineStr"/>
       <c r="M597" s="6" t="inlineStr"/>
     </row>
     <row r="598">
@@ -26393,21 +26403,21 @@
     <row r="599">
       <c r="A599" s="6" t="inlineStr">
         <is>
-          <t>SMRVA</t>
+          <t>AAGYO</t>
         </is>
       </c>
       <c r="B599" s="7" t="n">
-        <v>19.36</v>
+        <v>18.37</v>
       </c>
       <c r="C599" s="8" t="n">
-        <v>-0.0759</v>
+        <v>-0.0113</v>
       </c>
       <c r="D599" s="9" t="n">
-        <v>84430000</v>
+        <v>50560000</v>
       </c>
       <c r="E599" s="6" t="inlineStr"/>
       <c r="F599" s="7" t="n">
-        <v>59.13</v>
+        <v>27.15</v>
       </c>
       <c r="G599" s="6" t="inlineStr"/>
       <c r="H599" s="6" t="inlineStr"/>
@@ -26415,12 +26425,12 @@
       <c r="J599" s="6" t="inlineStr"/>
       <c r="K599" s="6" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L599" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M599" s="6" t="inlineStr"/>
@@ -26428,21 +26438,21 @@
     <row r="600">
       <c r="A600" s="2" t="inlineStr">
         <is>
-          <t>EMPAE</t>
+          <t>BESTE</t>
         </is>
       </c>
       <c r="B600" s="3" t="n">
-        <v>42.98</v>
+        <v>29.22</v>
       </c>
       <c r="C600" s="4" t="n">
-        <v>0.0998</v>
+        <v>-0.0214</v>
       </c>
       <c r="D600" s="5" t="n">
-        <v>11900000</v>
+        <v>22260000</v>
       </c>
       <c r="E600" s="2" t="inlineStr"/>
       <c r="F600" s="3" t="n">
-        <v>59.61</v>
+        <v>67.41</v>
       </c>
       <c r="G600" s="2" t="inlineStr"/>
       <c r="H600" s="2" t="inlineStr"/>
@@ -26450,12 +26460,12 @@
       <c r="J600" s="2" t="inlineStr"/>
       <c r="K600" s="2" t="inlineStr">
         <is>
-          <t>Elektronik teknoloji</t>
+          <t>Elektrik, Su, Gaz Hizmetleri</t>
         </is>
       </c>
       <c r="L600" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M600" s="2" t="inlineStr"/>
@@ -26463,26 +26473,32 @@
     <row r="601">
       <c r="A601" s="6" t="inlineStr">
         <is>
-          <t>AAGYO</t>
+          <t>BORLS</t>
         </is>
       </c>
       <c r="B601" s="7" t="n">
-        <v>18.37</v>
+        <v>8.81</v>
       </c>
       <c r="C601" s="8" t="n">
-        <v>-0.0113</v>
+        <v>0.0513</v>
       </c>
       <c r="D601" s="9" t="n">
-        <v>50560000</v>
-      </c>
-      <c r="E601" s="6" t="inlineStr"/>
+        <v>106140000</v>
+      </c>
+      <c r="E601" s="8" t="n">
+        <v>0.1672</v>
+      </c>
       <c r="F601" s="7" t="n">
-        <v>27.15</v>
+        <v>75.73</v>
       </c>
       <c r="G601" s="6" t="inlineStr"/>
       <c r="H601" s="6" t="inlineStr"/>
-      <c r="I601" s="6" t="inlineStr"/>
-      <c r="J601" s="6" t="inlineStr"/>
+      <c r="I601" s="8" t="n">
+        <v>-5.3262</v>
+      </c>
+      <c r="J601" s="8" t="n">
+        <v>-4.2562</v>
+      </c>
       <c r="K601" s="6" t="inlineStr">
         <is>
           <t>Finans</t>
@@ -26490,7 +26506,7 @@
       </c>
       <c r="L601" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M601" s="6" t="inlineStr"/>
@@ -26498,23 +26514,21 @@
     <row r="602">
       <c r="A602" s="2" t="inlineStr">
         <is>
-          <t>INTEK</t>
+          <t>GLRMK</t>
         </is>
       </c>
       <c r="B602" s="3" t="n">
-        <v>240.1</v>
+        <v>191</v>
       </c>
       <c r="C602" s="4" t="n">
-        <v>-0.0008</v>
-      </c>
-      <c r="D602" s="3" t="n">
-        <v>8029.999999999999</v>
-      </c>
-      <c r="E602" s="4" t="n">
-        <v>0.2578</v>
-      </c>
+        <v>0.0053</v>
+      </c>
+      <c r="D602" s="5" t="n">
+        <v>18010000</v>
+      </c>
+      <c r="E602" s="2" t="inlineStr"/>
       <c r="F602" s="3" t="n">
-        <v>40.66</v>
+        <v>45.76</v>
       </c>
       <c r="G602" s="2" t="inlineStr"/>
       <c r="H602" s="2" t="inlineStr"/>
@@ -26522,41 +26536,41 @@
       <c r="J602" s="2" t="inlineStr"/>
       <c r="K602" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L602" s="2" t="inlineStr"/>
+          <t>Endüstriyel hizmetler</t>
+        </is>
+      </c>
+      <c r="L602" s="2" t="inlineStr">
+        <is>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+        </is>
+      </c>
       <c r="M602" s="2" t="inlineStr"/>
     </row>
     <row r="603">
       <c r="A603" s="6" t="inlineStr">
         <is>
-          <t>BORLS</t>
+          <t>ICUGS</t>
         </is>
       </c>
       <c r="B603" s="7" t="n">
-        <v>8.81</v>
+        <v>6.07</v>
       </c>
       <c r="C603" s="8" t="n">
-        <v>0.0513</v>
+        <v>-0.0272</v>
       </c>
       <c r="D603" s="9" t="n">
-        <v>106140000</v>
+        <v>58970000</v>
       </c>
       <c r="E603" s="8" t="n">
-        <v>0.1672</v>
+        <v>0.8667</v>
       </c>
       <c r="F603" s="7" t="n">
-        <v>75.73</v>
+        <v>82.51000000000001</v>
       </c>
       <c r="G603" s="6" t="inlineStr"/>
       <c r="H603" s="6" t="inlineStr"/>
-      <c r="I603" s="8" t="n">
-        <v>-5.3262</v>
-      </c>
-      <c r="J603" s="8" t="n">
-        <v>-4.2562</v>
-      </c>
+      <c r="I603" s="6" t="inlineStr"/>
+      <c r="J603" s="6" t="inlineStr"/>
       <c r="K603" s="6" t="inlineStr">
         <is>
           <t>Finans</t>
@@ -26564,7 +26578,7 @@
       </c>
       <c r="L603" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
         </is>
       </c>
       <c r="M603" s="6" t="inlineStr"/>
@@ -26572,21 +26586,23 @@
     <row r="604">
       <c r="A604" s="2" t="inlineStr">
         <is>
-          <t>BESTE</t>
+          <t>UCAYM</t>
         </is>
       </c>
       <c r="B604" s="3" t="n">
-        <v>29.22</v>
+        <v>29.8</v>
       </c>
       <c r="C604" s="4" t="n">
-        <v>-0.0214</v>
-      </c>
-      <c r="D604" s="5" t="n">
-        <v>22260000</v>
-      </c>
-      <c r="E604" s="2" t="inlineStr"/>
+        <v>-0.0132</v>
+      </c>
+      <c r="D604" s="3" t="n">
+        <v>16620000</v>
+      </c>
+      <c r="E604" s="4" t="n">
+        <v>0.2667</v>
+      </c>
       <c r="F604" s="3" t="n">
-        <v>67.41</v>
+        <v>54.67</v>
       </c>
       <c r="G604" s="2" t="inlineStr"/>
       <c r="H604" s="2" t="inlineStr"/>
@@ -26594,12 +26610,12 @@
       <c r="J604" s="2" t="inlineStr"/>
       <c r="K604" s="2" t="inlineStr">
         <is>
-          <t>Elektrik, Su, Gaz Hizmetleri</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L604" s="2" t="inlineStr">
         <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M604" s="2" t="inlineStr"/>
@@ -26607,93 +26623,91 @@
     <row r="605">
       <c r="A605" s="6" t="inlineStr">
         <is>
-          <t>ALTIN</t>
+          <t>BRMEN</t>
         </is>
       </c>
       <c r="B605" s="7" t="n">
-        <v>79.78</v>
+        <v>6.75</v>
       </c>
       <c r="C605" s="8" t="n">
-        <v>0.0036</v>
+        <v>0.0433</v>
       </c>
       <c r="D605" s="9" t="n">
-        <v>9710000</v>
-      </c>
-      <c r="E605" s="6" t="inlineStr"/>
+        <v>707270</v>
+      </c>
+      <c r="E605" s="8" t="n">
+        <v>0.95</v>
+      </c>
       <c r="F605" s="7" t="n">
-        <v>41.39</v>
+        <v>37.16</v>
       </c>
       <c r="G605" s="6" t="inlineStr"/>
       <c r="H605" s="6" t="inlineStr"/>
-      <c r="I605" s="6" t="inlineStr"/>
-      <c r="J605" s="6" t="inlineStr"/>
-      <c r="K605" s="6" t="inlineStr"/>
+      <c r="I605" s="8" t="n">
+        <v>-23.6291</v>
+      </c>
+      <c r="J605" s="8" t="n">
+        <v>-0.4678</v>
+      </c>
+      <c r="K605" s="6" t="inlineStr">
+        <is>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
       <c r="L605" s="6" t="inlineStr"/>
       <c r="M605" s="6" t="inlineStr"/>
     </row>
     <row r="606">
       <c r="A606" s="2" t="inlineStr">
         <is>
-          <t>BERA</t>
+          <t>DMLKT</t>
         </is>
       </c>
       <c r="B606" s="3" t="n">
-        <v>17.35</v>
+        <v>6.15</v>
       </c>
       <c r="C606" s="4" t="n">
-        <v>0.014</v>
+        <v>-0.0032</v>
       </c>
       <c r="D606" s="5" t="n">
-        <v>11300000</v>
-      </c>
-      <c r="E606" s="4" t="n">
-        <v>0.9246</v>
-      </c>
+        <v>6880000</v>
+      </c>
+      <c r="E606" s="2" t="inlineStr"/>
       <c r="F606" s="3" t="n">
-        <v>50.67</v>
-      </c>
-      <c r="G606" s="3" t="n">
-        <v>163.99</v>
-      </c>
+        <v>60.46</v>
+      </c>
+      <c r="G606" s="2" t="inlineStr"/>
       <c r="H606" s="2" t="inlineStr"/>
-      <c r="I606" s="4" t="n">
-        <v>0.0028</v>
-      </c>
-      <c r="J606" s="4" t="n">
-        <v>-10.3171</v>
-      </c>
+      <c r="I606" s="2" t="inlineStr"/>
+      <c r="J606" s="2" t="inlineStr"/>
       <c r="K606" s="2" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
-        </is>
-      </c>
-      <c r="L606" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KONYA</t>
-        </is>
-      </c>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L606" s="2" t="inlineStr"/>
       <c r="M606" s="2" t="inlineStr"/>
     </row>
     <row r="607">
       <c r="A607" s="6" t="inlineStr">
         <is>
-          <t>UCAYM</t>
+          <t>INTEK</t>
         </is>
       </c>
       <c r="B607" s="7" t="n">
-        <v>29.8</v>
+        <v>240.1</v>
       </c>
       <c r="C607" s="8" t="n">
-        <v>-0.0132</v>
+        <v>-0.0008</v>
       </c>
       <c r="D607" s="7" t="n">
-        <v>16620000</v>
+        <v>8029.999999999999</v>
       </c>
       <c r="E607" s="8" t="n">
-        <v>0.2667</v>
+        <v>0.2578</v>
       </c>
       <c r="F607" s="7" t="n">
-        <v>54.67</v>
+        <v>40.66</v>
       </c>
       <c r="G607" s="6" t="inlineStr"/>
       <c r="H607" s="6" t="inlineStr"/>
@@ -26701,34 +26715,30 @@
       <c r="J607" s="6" t="inlineStr"/>
       <c r="K607" s="6" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
-        </is>
-      </c>
-      <c r="L607" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L607" s="6" t="inlineStr"/>
       <c r="M607" s="6" t="inlineStr"/>
     </row>
     <row r="608">
       <c r="A608" s="2" t="inlineStr">
         <is>
-          <t>LXGYO</t>
+          <t>MARMR</t>
         </is>
       </c>
       <c r="B608" s="3" t="n">
-        <v>17.89</v>
+        <v>2.83</v>
       </c>
       <c r="C608" s="4" t="n">
-        <v>0.0371</v>
-      </c>
-      <c r="D608" s="3" t="n">
-        <v>66540000.00000001</v>
+        <v>-0.0174</v>
+      </c>
+      <c r="D608" s="5" t="n">
+        <v>210300000</v>
       </c>
       <c r="E608" s="2" t="inlineStr"/>
       <c r="F608" s="3" t="n">
-        <v>56.21</v>
+        <v>51.51</v>
       </c>
       <c r="G608" s="2" t="inlineStr"/>
       <c r="H608" s="2" t="inlineStr"/>
@@ -26741,7 +26751,7 @@
       </c>
       <c r="L608" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M608" s="2" t="inlineStr"/>
@@ -26749,34 +26759,40 @@
     <row r="609">
       <c r="A609" s="6" t="inlineStr">
         <is>
-          <t>MCARD</t>
+          <t>CRFSA</t>
         </is>
       </c>
       <c r="B609" s="7" t="n">
-        <v>178.6</v>
+        <v>147</v>
       </c>
       <c r="C609" s="8" t="n">
-        <v>0.0998</v>
+        <v>0.0138</v>
       </c>
       <c r="D609" s="9" t="n">
-        <v>6520000</v>
-      </c>
-      <c r="E609" s="6" t="inlineStr"/>
+        <v>2130000</v>
+      </c>
+      <c r="E609" s="8" t="n">
+        <v>0.1071</v>
+      </c>
       <c r="F609" s="7" t="n">
-        <v>62.69</v>
+        <v>50.74</v>
       </c>
       <c r="G609" s="6" t="inlineStr"/>
       <c r="H609" s="6" t="inlineStr"/>
-      <c r="I609" s="6" t="inlineStr"/>
-      <c r="J609" s="6" t="inlineStr"/>
+      <c r="I609" s="8" t="n">
+        <v>-3.6635</v>
+      </c>
+      <c r="J609" s="8" t="n">
+        <v>-0.4897</v>
+      </c>
       <c r="K609" s="6" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>Perakende satış</t>
         </is>
       </c>
       <c r="L609" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
         </is>
       </c>
       <c r="M609" s="6" t="inlineStr"/>
@@ -26784,40 +26800,34 @@
     <row r="610">
       <c r="A610" s="2" t="inlineStr">
         <is>
-          <t>CRFSA</t>
+          <t>FRMPL</t>
         </is>
       </c>
       <c r="B610" s="3" t="n">
-        <v>147</v>
+        <v>33.98</v>
       </c>
       <c r="C610" s="4" t="n">
-        <v>0.0138</v>
-      </c>
-      <c r="D610" s="5" t="n">
-        <v>2130000</v>
-      </c>
-      <c r="E610" s="4" t="n">
-        <v>0.1071</v>
-      </c>
+        <v>0.0253</v>
+      </c>
+      <c r="D610" s="3" t="n">
+        <v>4020000</v>
+      </c>
+      <c r="E610" s="2" t="inlineStr"/>
       <c r="F610" s="3" t="n">
-        <v>50.74</v>
+        <v>53.84</v>
       </c>
       <c r="G610" s="2" t="inlineStr"/>
       <c r="H610" s="2" t="inlineStr"/>
-      <c r="I610" s="4" t="n">
-        <v>-3.6635</v>
-      </c>
-      <c r="J610" s="4" t="n">
-        <v>-0.4897</v>
-      </c>
+      <c r="I610" s="2" t="inlineStr"/>
+      <c r="J610" s="2" t="inlineStr"/>
       <c r="K610" s="2" t="inlineStr">
         <is>
-          <t>Perakende satış</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L610" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M610" s="2" t="inlineStr"/>
@@ -26825,37 +26835,27 @@
     <row r="611">
       <c r="A611" s="6" t="inlineStr">
         <is>
-          <t>BRMEN</t>
+          <t>ALTIN</t>
         </is>
       </c>
       <c r="B611" s="7" t="n">
-        <v>6.75</v>
+        <v>79.78</v>
       </c>
       <c r="C611" s="8" t="n">
-        <v>0.0433</v>
+        <v>0.0036</v>
       </c>
       <c r="D611" s="9" t="n">
-        <v>707270</v>
-      </c>
-      <c r="E611" s="8" t="n">
-        <v>0.95</v>
-      </c>
+        <v>9710000</v>
+      </c>
+      <c r="E611" s="6" t="inlineStr"/>
       <c r="F611" s="7" t="n">
-        <v>37.16</v>
+        <v>41.39</v>
       </c>
       <c r="G611" s="6" t="inlineStr"/>
       <c r="H611" s="6" t="inlineStr"/>
-      <c r="I611" s="8" t="n">
-        <v>-23.6291</v>
-      </c>
-      <c r="J611" s="8" t="n">
-        <v>-0.4678</v>
-      </c>
-      <c r="K611" s="6" t="inlineStr">
-        <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
+      <c r="I611" s="6" t="inlineStr"/>
+      <c r="J611" s="6" t="inlineStr"/>
+      <c r="K611" s="6" t="inlineStr"/>
       <c r="L611" s="6" t="inlineStr"/>
       <c r="M611" s="6" t="inlineStr"/>
     </row>
@@ -26881,7 +26881,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>05.05.2026 16:30</t>
+          <t>05.05.2026 17:02</t>
         </is>
       </c>
     </row>

</xml_diff>